<commit_message>
Add weighed cylinder mass and mass loss matching supplied register
</commit_message>
<xml_diff>
--- a/resources/templates/cylinder-import.xlsx
+++ b/resources/templates/cylinder-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Urządzenia" sheetId="1" r:id="Rb7beff886c3443f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrukcja" sheetId="2" r:id="R67cefbb5257743c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Urządzenia" sheetId="1" r:id="R1343976b27c54540"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrukcja" sheetId="2" r:id="Rd2d560a8fa35401f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,12 +55,22 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1A4D3A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1A4D3A"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -80,7 +90,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -104,6 +114,20 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -325,64 +349,72 @@
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="64" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+    <x:row r="1" ht="80" customHeight="1">
+      <x:c r="A1" s="20" t="str">
         <x:v>Nazwa urządzenia</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
-        <x:v>Znak wytwórczy</x:v>
+      <x:c r="B1" s="20" t="str">
+        <x:v>Nazwa lub znak wytwórcy</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="20" t="str">
         <x:v>Rok produkcji</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="20" t="str">
         <x:v>Numer fabryczny</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="20" t="str">
         <x:v>Numer ewidencyjny u eksploatującego</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="20" t="str">
         <x:v>Czynnik roboczy</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="20" t="str">
         <x:v>Temperatura dopuszczalna min. [°C]</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="20" t="str">
         <x:v>Temperatura dopuszczalna max. [°C]</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="I1" s="20" t="str">
         <x:v>Pojemność [dm³]</x:v>
       </x:c>
-      <x:c r="J1" s="6" t="str">
+      <x:c r="J1" s="20" t="str">
         <x:v>Ciśnienie robocze [bar]</x:v>
       </x:c>
-      <x:c r="K1" s="6" t="str">
+      <x:c r="K1" s="20" t="str">
         <x:v>Ciśnienie próbne [bar]</x:v>
       </x:c>
-      <x:c r="L1" s="6" t="str">
+      <x:c r="L1" s="20" t="str">
         <x:v>Tara lub masa brutto [kg]</x:v>
       </x:c>
-      <x:c r="M1" s="6" t="str">
+      <x:c r="M1" s="20" t="str">
         <x:v>Masa netto [kg]</x:v>
       </x:c>
-      <x:c r="N1" s="6" t="str">
+      <x:c r="N1" s="20" t="str">
         <x:v>Masa butli bez osprzętu — wybita [kg]</x:v>
       </x:c>
-      <x:c r="O1" s="6" t="str">
-        <x:v>Symbol masy przewożonej / dopuszczalnej</x:v>
+      <x:c r="O1" s="20" t="str">
+        <x:v>Masa butli bez osprzętu — według ważenia [kg]</x:v>
       </x:c>
-      <x:c r="P1" s="6" t="str">
+      <x:c r="P1" s="20" t="str">
+        <x:v>Masa butli bez osprzętu — ubytek [kg]</x:v>
+      </x:c>
+      <x:c r="Q1" s="20" t="str">
+        <x:v>Symbol masy prowizorycznej / rozpuszczalnika</x:v>
+      </x:c>
+      <x:c r="R1" s="20" t="str">
         <x:v>Osprzęt — typ</x:v>
       </x:c>
-      <x:c r="Q1" s="6" t="str">
-        <x:v>Osprzęt — znak Π lub CE</x:v>
+      <x:c r="S1" s="20" t="str">
+        <x:v>Osprzęt — znak II lub CE</x:v>
       </x:c>
-      <x:c r="R1" s="6" t="str">
+      <x:c r="T1" s="20" t="str">
         <x:v>Producent (informacja dodatkowa)</x:v>
       </x:c>
-      <x:c r="S1" s="6" t="str">
+      <x:c r="U1" s="20" t="str">
         <x:v>Uwagi</x:v>
       </x:c>
     </x:row>
@@ -401,11 +433,13 @@
       <x:c r="L2" s="9"/>
       <x:c r="M2" s="9"/>
       <x:c r="N2" s="9"/>
-      <x:c r="O2" s="8"/>
-      <x:c r="P2" s="8"/>
+      <x:c r="O2" s="9"/>
+      <x:c r="P2" s="9"/>
       <x:c r="Q2" s="8"/>
       <x:c r="R2" s="8"/>
       <x:c r="S2" s="8"/>
+      <x:c r="T2" s="8"/>
+      <x:c r="U2" s="8"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="8"/>
@@ -422,11 +456,13 @@
       <x:c r="L3" s="9"/>
       <x:c r="M3" s="9"/>
       <x:c r="N3" s="9"/>
-      <x:c r="O3" s="8"/>
-      <x:c r="P3" s="8"/>
+      <x:c r="O3" s="9"/>
+      <x:c r="P3" s="9"/>
       <x:c r="Q3" s="8"/>
       <x:c r="R3" s="8"/>
       <x:c r="S3" s="8"/>
+      <x:c r="T3" s="8"/>
+      <x:c r="U3" s="8"/>
     </x:row>
     <x:row r="4" ht="20" customHeight="1">
       <x:c r="A4" s="8"/>
@@ -443,11 +479,13 @@
       <x:c r="L4" s="9"/>
       <x:c r="M4" s="9"/>
       <x:c r="N4" s="9"/>
-      <x:c r="O4" s="8"/>
-      <x:c r="P4" s="8"/>
+      <x:c r="O4" s="9"/>
+      <x:c r="P4" s="9"/>
       <x:c r="Q4" s="8"/>
       <x:c r="R4" s="8"/>
       <x:c r="S4" s="8"/>
+      <x:c r="T4" s="8"/>
+      <x:c r="U4" s="8"/>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="8"/>
@@ -464,11 +502,13 @@
       <x:c r="L5" s="9"/>
       <x:c r="M5" s="9"/>
       <x:c r="N5" s="9"/>
-      <x:c r="O5" s="8"/>
-      <x:c r="P5" s="8"/>
+      <x:c r="O5" s="9"/>
+      <x:c r="P5" s="9"/>
       <x:c r="Q5" s="8"/>
       <x:c r="R5" s="8"/>
       <x:c r="S5" s="8"/>
+      <x:c r="T5" s="8"/>
+      <x:c r="U5" s="8"/>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="8"/>
@@ -485,11 +525,13 @@
       <x:c r="L6" s="9"/>
       <x:c r="M6" s="9"/>
       <x:c r="N6" s="9"/>
-      <x:c r="O6" s="8"/>
-      <x:c r="P6" s="8"/>
+      <x:c r="O6" s="9"/>
+      <x:c r="P6" s="9"/>
       <x:c r="Q6" s="8"/>
       <x:c r="R6" s="8"/>
       <x:c r="S6" s="8"/>
+      <x:c r="T6" s="8"/>
+      <x:c r="U6" s="8"/>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="8"/>
@@ -506,11 +548,13 @@
       <x:c r="L7" s="9"/>
       <x:c r="M7" s="9"/>
       <x:c r="N7" s="9"/>
-      <x:c r="O7" s="8"/>
-      <x:c r="P7" s="8"/>
+      <x:c r="O7" s="9"/>
+      <x:c r="P7" s="9"/>
       <x:c r="Q7" s="8"/>
       <x:c r="R7" s="8"/>
       <x:c r="S7" s="8"/>
+      <x:c r="T7" s="8"/>
+      <x:c r="U7" s="8"/>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="8"/>
@@ -527,11 +571,13 @@
       <x:c r="L8" s="9"/>
       <x:c r="M8" s="9"/>
       <x:c r="N8" s="9"/>
-      <x:c r="O8" s="8"/>
-      <x:c r="P8" s="8"/>
+      <x:c r="O8" s="9"/>
+      <x:c r="P8" s="9"/>
       <x:c r="Q8" s="8"/>
       <x:c r="R8" s="8"/>
       <x:c r="S8" s="8"/>
+      <x:c r="T8" s="8"/>
+      <x:c r="U8" s="8"/>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="8"/>
@@ -548,11 +594,13 @@
       <x:c r="L9" s="9"/>
       <x:c r="M9" s="9"/>
       <x:c r="N9" s="9"/>
-      <x:c r="O9" s="8"/>
-      <x:c r="P9" s="8"/>
+      <x:c r="O9" s="9"/>
+      <x:c r="P9" s="9"/>
       <x:c r="Q9" s="8"/>
       <x:c r="R9" s="8"/>
       <x:c r="S9" s="8"/>
+      <x:c r="T9" s="8"/>
+      <x:c r="U9" s="8"/>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="8"/>
@@ -569,11 +617,13 @@
       <x:c r="L10" s="9"/>
       <x:c r="M10" s="9"/>
       <x:c r="N10" s="9"/>
-      <x:c r="O10" s="8"/>
-      <x:c r="P10" s="8"/>
+      <x:c r="O10" s="9"/>
+      <x:c r="P10" s="9"/>
       <x:c r="Q10" s="8"/>
       <x:c r="R10" s="8"/>
       <x:c r="S10" s="8"/>
+      <x:c r="T10" s="8"/>
+      <x:c r="U10" s="8"/>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="8"/>
@@ -590,11 +640,13 @@
       <x:c r="L11" s="9"/>
       <x:c r="M11" s="9"/>
       <x:c r="N11" s="9"/>
-      <x:c r="O11" s="8"/>
-      <x:c r="P11" s="8"/>
+      <x:c r="O11" s="9"/>
+      <x:c r="P11" s="9"/>
       <x:c r="Q11" s="8"/>
       <x:c r="R11" s="8"/>
       <x:c r="S11" s="8"/>
+      <x:c r="T11" s="8"/>
+      <x:c r="U11" s="8"/>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
       <x:c r="A12" s="8"/>
@@ -611,11 +663,13 @@
       <x:c r="L12" s="9"/>
       <x:c r="M12" s="9"/>
       <x:c r="N12" s="9"/>
-      <x:c r="O12" s="8"/>
-      <x:c r="P12" s="8"/>
+      <x:c r="O12" s="9"/>
+      <x:c r="P12" s="9"/>
       <x:c r="Q12" s="8"/>
       <x:c r="R12" s="8"/>
       <x:c r="S12" s="8"/>
+      <x:c r="T12" s="8"/>
+      <x:c r="U12" s="8"/>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
       <x:c r="A13" s="8"/>
@@ -632,11 +686,13 @@
       <x:c r="L13" s="9"/>
       <x:c r="M13" s="9"/>
       <x:c r="N13" s="9"/>
-      <x:c r="O13" s="8"/>
-      <x:c r="P13" s="8"/>
+      <x:c r="O13" s="9"/>
+      <x:c r="P13" s="9"/>
       <x:c r="Q13" s="8"/>
       <x:c r="R13" s="8"/>
       <x:c r="S13" s="8"/>
+      <x:c r="T13" s="8"/>
+      <x:c r="U13" s="8"/>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
       <x:c r="A14" s="8"/>
@@ -653,11 +709,13 @@
       <x:c r="L14" s="9"/>
       <x:c r="M14" s="9"/>
       <x:c r="N14" s="9"/>
-      <x:c r="O14" s="8"/>
-      <x:c r="P14" s="8"/>
+      <x:c r="O14" s="9"/>
+      <x:c r="P14" s="9"/>
       <x:c r="Q14" s="8"/>
       <x:c r="R14" s="8"/>
       <x:c r="S14" s="8"/>
+      <x:c r="T14" s="8"/>
+      <x:c r="U14" s="8"/>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
       <x:c r="A15" s="8"/>
@@ -674,11 +732,13 @@
       <x:c r="L15" s="9"/>
       <x:c r="M15" s="9"/>
       <x:c r="N15" s="9"/>
-      <x:c r="O15" s="8"/>
-      <x:c r="P15" s="8"/>
+      <x:c r="O15" s="9"/>
+      <x:c r="P15" s="9"/>
       <x:c r="Q15" s="8"/>
       <x:c r="R15" s="8"/>
       <x:c r="S15" s="8"/>
+      <x:c r="T15" s="8"/>
+      <x:c r="U15" s="8"/>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
       <x:c r="A16" s="8"/>
@@ -695,11 +755,13 @@
       <x:c r="L16" s="9"/>
       <x:c r="M16" s="9"/>
       <x:c r="N16" s="9"/>
-      <x:c r="O16" s="8"/>
-      <x:c r="P16" s="8"/>
+      <x:c r="O16" s="9"/>
+      <x:c r="P16" s="9"/>
       <x:c r="Q16" s="8"/>
       <x:c r="R16" s="8"/>
       <x:c r="S16" s="8"/>
+      <x:c r="T16" s="8"/>
+      <x:c r="U16" s="8"/>
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
       <x:c r="A17" s="8"/>
@@ -716,11 +778,13 @@
       <x:c r="L17" s="9"/>
       <x:c r="M17" s="9"/>
       <x:c r="N17" s="9"/>
-      <x:c r="O17" s="8"/>
-      <x:c r="P17" s="8"/>
+      <x:c r="O17" s="9"/>
+      <x:c r="P17" s="9"/>
       <x:c r="Q17" s="8"/>
       <x:c r="R17" s="8"/>
       <x:c r="S17" s="8"/>
+      <x:c r="T17" s="8"/>
+      <x:c r="U17" s="8"/>
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
       <x:c r="A18" s="8"/>
@@ -737,11 +801,13 @@
       <x:c r="L18" s="9"/>
       <x:c r="M18" s="9"/>
       <x:c r="N18" s="9"/>
-      <x:c r="O18" s="8"/>
-      <x:c r="P18" s="8"/>
+      <x:c r="O18" s="9"/>
+      <x:c r="P18" s="9"/>
       <x:c r="Q18" s="8"/>
       <x:c r="R18" s="8"/>
       <x:c r="S18" s="8"/>
+      <x:c r="T18" s="8"/>
+      <x:c r="U18" s="8"/>
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
       <x:c r="A19" s="8"/>
@@ -758,11 +824,13 @@
       <x:c r="L19" s="9"/>
       <x:c r="M19" s="9"/>
       <x:c r="N19" s="9"/>
-      <x:c r="O19" s="8"/>
-      <x:c r="P19" s="8"/>
+      <x:c r="O19" s="9"/>
+      <x:c r="P19" s="9"/>
       <x:c r="Q19" s="8"/>
       <x:c r="R19" s="8"/>
       <x:c r="S19" s="8"/>
+      <x:c r="T19" s="8"/>
+      <x:c r="U19" s="8"/>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
       <x:c r="A20" s="8"/>
@@ -779,11 +847,13 @@
       <x:c r="L20" s="9"/>
       <x:c r="M20" s="9"/>
       <x:c r="N20" s="9"/>
-      <x:c r="O20" s="8"/>
-      <x:c r="P20" s="8"/>
+      <x:c r="O20" s="9"/>
+      <x:c r="P20" s="9"/>
       <x:c r="Q20" s="8"/>
       <x:c r="R20" s="8"/>
       <x:c r="S20" s="8"/>
+      <x:c r="T20" s="8"/>
+      <x:c r="U20" s="8"/>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
       <x:c r="A21" s="8"/>
@@ -800,11 +870,13 @@
       <x:c r="L21" s="9"/>
       <x:c r="M21" s="9"/>
       <x:c r="N21" s="9"/>
-      <x:c r="O21" s="8"/>
-      <x:c r="P21" s="8"/>
+      <x:c r="O21" s="9"/>
+      <x:c r="P21" s="9"/>
       <x:c r="Q21" s="8"/>
       <x:c r="R21" s="8"/>
       <x:c r="S21" s="8"/>
+      <x:c r="T21" s="8"/>
+      <x:c r="U21" s="8"/>
     </x:row>
     <x:row r="22" ht="20" customHeight="1">
       <x:c r="A22" s="8"/>
@@ -821,11 +893,13 @@
       <x:c r="L22" s="9"/>
       <x:c r="M22" s="9"/>
       <x:c r="N22" s="9"/>
-      <x:c r="O22" s="8"/>
-      <x:c r="P22" s="8"/>
+      <x:c r="O22" s="9"/>
+      <x:c r="P22" s="9"/>
       <x:c r="Q22" s="8"/>
       <x:c r="R22" s="8"/>
       <x:c r="S22" s="8"/>
+      <x:c r="T22" s="8"/>
+      <x:c r="U22" s="8"/>
     </x:row>
     <x:row r="23" ht="20" customHeight="1">
       <x:c r="A23" s="8"/>
@@ -842,11 +916,13 @@
       <x:c r="L23" s="9"/>
       <x:c r="M23" s="9"/>
       <x:c r="N23" s="9"/>
-      <x:c r="O23" s="8"/>
-      <x:c r="P23" s="8"/>
+      <x:c r="O23" s="9"/>
+      <x:c r="P23" s="9"/>
       <x:c r="Q23" s="8"/>
       <x:c r="R23" s="8"/>
       <x:c r="S23" s="8"/>
+      <x:c r="T23" s="8"/>
+      <x:c r="U23" s="8"/>
     </x:row>
     <x:row r="24" ht="20" customHeight="1">
       <x:c r="A24" s="8"/>
@@ -863,11 +939,13 @@
       <x:c r="L24" s="9"/>
       <x:c r="M24" s="9"/>
       <x:c r="N24" s="9"/>
-      <x:c r="O24" s="8"/>
-      <x:c r="P24" s="8"/>
+      <x:c r="O24" s="9"/>
+      <x:c r="P24" s="9"/>
       <x:c r="Q24" s="8"/>
       <x:c r="R24" s="8"/>
       <x:c r="S24" s="8"/>
+      <x:c r="T24" s="8"/>
+      <x:c r="U24" s="8"/>
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
       <x:c r="A25" s="8"/>
@@ -884,11 +962,13 @@
       <x:c r="L25" s="9"/>
       <x:c r="M25" s="9"/>
       <x:c r="N25" s="9"/>
-      <x:c r="O25" s="8"/>
-      <x:c r="P25" s="8"/>
+      <x:c r="O25" s="9"/>
+      <x:c r="P25" s="9"/>
       <x:c r="Q25" s="8"/>
       <x:c r="R25" s="8"/>
       <x:c r="S25" s="8"/>
+      <x:c r="T25" s="8"/>
+      <x:c r="U25" s="8"/>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
       <x:c r="A26" s="8"/>
@@ -905,11 +985,13 @@
       <x:c r="L26" s="9"/>
       <x:c r="M26" s="9"/>
       <x:c r="N26" s="9"/>
-      <x:c r="O26" s="8"/>
-      <x:c r="P26" s="8"/>
+      <x:c r="O26" s="9"/>
+      <x:c r="P26" s="9"/>
       <x:c r="Q26" s="8"/>
       <x:c r="R26" s="8"/>
       <x:c r="S26" s="8"/>
+      <x:c r="T26" s="8"/>
+      <x:c r="U26" s="8"/>
     </x:row>
     <x:row r="27" ht="20" customHeight="1">
       <x:c r="A27" s="8"/>
@@ -926,11 +1008,13 @@
       <x:c r="L27" s="9"/>
       <x:c r="M27" s="9"/>
       <x:c r="N27" s="9"/>
-      <x:c r="O27" s="8"/>
-      <x:c r="P27" s="8"/>
+      <x:c r="O27" s="9"/>
+      <x:c r="P27" s="9"/>
       <x:c r="Q27" s="8"/>
       <x:c r="R27" s="8"/>
       <x:c r="S27" s="8"/>
+      <x:c r="T27" s="8"/>
+      <x:c r="U27" s="8"/>
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
       <x:c r="A28" s="8"/>
@@ -947,11 +1031,13 @@
       <x:c r="L28" s="9"/>
       <x:c r="M28" s="9"/>
       <x:c r="N28" s="9"/>
-      <x:c r="O28" s="8"/>
-      <x:c r="P28" s="8"/>
+      <x:c r="O28" s="9"/>
+      <x:c r="P28" s="9"/>
       <x:c r="Q28" s="8"/>
       <x:c r="R28" s="8"/>
       <x:c r="S28" s="8"/>
+      <x:c r="T28" s="8"/>
+      <x:c r="U28" s="8"/>
     </x:row>
     <x:row r="29" ht="20" customHeight="1">
       <x:c r="A29" s="8"/>
@@ -968,11 +1054,13 @@
       <x:c r="L29" s="9"/>
       <x:c r="M29" s="9"/>
       <x:c r="N29" s="9"/>
-      <x:c r="O29" s="8"/>
-      <x:c r="P29" s="8"/>
+      <x:c r="O29" s="9"/>
+      <x:c r="P29" s="9"/>
       <x:c r="Q29" s="8"/>
       <x:c r="R29" s="8"/>
       <x:c r="S29" s="8"/>
+      <x:c r="T29" s="8"/>
+      <x:c r="U29" s="8"/>
     </x:row>
     <x:row r="30" ht="20" customHeight="1">
       <x:c r="A30" s="8"/>
@@ -989,11 +1077,13 @@
       <x:c r="L30" s="9"/>
       <x:c r="M30" s="9"/>
       <x:c r="N30" s="9"/>
-      <x:c r="O30" s="8"/>
-      <x:c r="P30" s="8"/>
+      <x:c r="O30" s="9"/>
+      <x:c r="P30" s="9"/>
       <x:c r="Q30" s="8"/>
       <x:c r="R30" s="8"/>
       <x:c r="S30" s="8"/>
+      <x:c r="T30" s="8"/>
+      <x:c r="U30" s="8"/>
     </x:row>
     <x:row r="31" ht="20" customHeight="1">
       <x:c r="A31" s="8"/>
@@ -1010,11 +1100,13 @@
       <x:c r="L31" s="9"/>
       <x:c r="M31" s="9"/>
       <x:c r="N31" s="9"/>
-      <x:c r="O31" s="8"/>
-      <x:c r="P31" s="8"/>
+      <x:c r="O31" s="9"/>
+      <x:c r="P31" s="9"/>
       <x:c r="Q31" s="8"/>
       <x:c r="R31" s="8"/>
       <x:c r="S31" s="8"/>
+      <x:c r="T31" s="8"/>
+      <x:c r="U31" s="8"/>
     </x:row>
     <x:row r="32" ht="20" customHeight="1">
       <x:c r="A32" s="8"/>
@@ -1031,11 +1123,13 @@
       <x:c r="L32" s="9"/>
       <x:c r="M32" s="9"/>
       <x:c r="N32" s="9"/>
-      <x:c r="O32" s="8"/>
-      <x:c r="P32" s="8"/>
+      <x:c r="O32" s="9"/>
+      <x:c r="P32" s="9"/>
       <x:c r="Q32" s="8"/>
       <x:c r="R32" s="8"/>
       <x:c r="S32" s="8"/>
+      <x:c r="T32" s="8"/>
+      <x:c r="U32" s="8"/>
     </x:row>
     <x:row r="33" ht="20" customHeight="1">
       <x:c r="A33" s="8"/>
@@ -1052,11 +1146,13 @@
       <x:c r="L33" s="9"/>
       <x:c r="M33" s="9"/>
       <x:c r="N33" s="9"/>
-      <x:c r="O33" s="8"/>
-      <x:c r="P33" s="8"/>
+      <x:c r="O33" s="9"/>
+      <x:c r="P33" s="9"/>
       <x:c r="Q33" s="8"/>
       <x:c r="R33" s="8"/>
       <x:c r="S33" s="8"/>
+      <x:c r="T33" s="8"/>
+      <x:c r="U33" s="8"/>
     </x:row>
     <x:row r="34" ht="20" customHeight="1">
       <x:c r="A34" s="8"/>
@@ -1073,11 +1169,13 @@
       <x:c r="L34" s="9"/>
       <x:c r="M34" s="9"/>
       <x:c r="N34" s="9"/>
-      <x:c r="O34" s="8"/>
-      <x:c r="P34" s="8"/>
+      <x:c r="O34" s="9"/>
+      <x:c r="P34" s="9"/>
       <x:c r="Q34" s="8"/>
       <x:c r="R34" s="8"/>
       <x:c r="S34" s="8"/>
+      <x:c r="T34" s="8"/>
+      <x:c r="U34" s="8"/>
     </x:row>
     <x:row r="35" ht="20" customHeight="1">
       <x:c r="A35" s="8"/>
@@ -1094,11 +1192,13 @@
       <x:c r="L35" s="9"/>
       <x:c r="M35" s="9"/>
       <x:c r="N35" s="9"/>
-      <x:c r="O35" s="8"/>
-      <x:c r="P35" s="8"/>
+      <x:c r="O35" s="9"/>
+      <x:c r="P35" s="9"/>
       <x:c r="Q35" s="8"/>
       <x:c r="R35" s="8"/>
       <x:c r="S35" s="8"/>
+      <x:c r="T35" s="8"/>
+      <x:c r="U35" s="8"/>
     </x:row>
     <x:row r="36" ht="20" customHeight="1">
       <x:c r="A36" s="8"/>
@@ -1115,11 +1215,13 @@
       <x:c r="L36" s="9"/>
       <x:c r="M36" s="9"/>
       <x:c r="N36" s="9"/>
-      <x:c r="O36" s="8"/>
-      <x:c r="P36" s="8"/>
+      <x:c r="O36" s="9"/>
+      <x:c r="P36" s="9"/>
       <x:c r="Q36" s="8"/>
       <x:c r="R36" s="8"/>
       <x:c r="S36" s="8"/>
+      <x:c r="T36" s="8"/>
+      <x:c r="U36" s="8"/>
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
       <x:c r="A37" s="8"/>
@@ -1136,11 +1238,13 @@
       <x:c r="L37" s="9"/>
       <x:c r="M37" s="9"/>
       <x:c r="N37" s="9"/>
-      <x:c r="O37" s="8"/>
-      <x:c r="P37" s="8"/>
+      <x:c r="O37" s="9"/>
+      <x:c r="P37" s="9"/>
       <x:c r="Q37" s="8"/>
       <x:c r="R37" s="8"/>
       <x:c r="S37" s="8"/>
+      <x:c r="T37" s="8"/>
+      <x:c r="U37" s="8"/>
     </x:row>
     <x:row r="38" ht="20" customHeight="1">
       <x:c r="A38" s="8"/>
@@ -1157,11 +1261,13 @@
       <x:c r="L38" s="9"/>
       <x:c r="M38" s="9"/>
       <x:c r="N38" s="9"/>
-      <x:c r="O38" s="8"/>
-      <x:c r="P38" s="8"/>
+      <x:c r="O38" s="9"/>
+      <x:c r="P38" s="9"/>
       <x:c r="Q38" s="8"/>
       <x:c r="R38" s="8"/>
       <x:c r="S38" s="8"/>
+      <x:c r="T38" s="8"/>
+      <x:c r="U38" s="8"/>
     </x:row>
     <x:row r="39" ht="20" customHeight="1">
       <x:c r="A39" s="8"/>
@@ -1178,11 +1284,13 @@
       <x:c r="L39" s="9"/>
       <x:c r="M39" s="9"/>
       <x:c r="N39" s="9"/>
-      <x:c r="O39" s="8"/>
-      <x:c r="P39" s="8"/>
+      <x:c r="O39" s="9"/>
+      <x:c r="P39" s="9"/>
       <x:c r="Q39" s="8"/>
       <x:c r="R39" s="8"/>
       <x:c r="S39" s="8"/>
+      <x:c r="T39" s="8"/>
+      <x:c r="U39" s="8"/>
     </x:row>
     <x:row r="40" ht="20" customHeight="1">
       <x:c r="A40" s="8"/>
@@ -1199,11 +1307,13 @@
       <x:c r="L40" s="9"/>
       <x:c r="M40" s="9"/>
       <x:c r="N40" s="9"/>
-      <x:c r="O40" s="8"/>
-      <x:c r="P40" s="8"/>
+      <x:c r="O40" s="9"/>
+      <x:c r="P40" s="9"/>
       <x:c r="Q40" s="8"/>
       <x:c r="R40" s="8"/>
       <x:c r="S40" s="8"/>
+      <x:c r="T40" s="8"/>
+      <x:c r="U40" s="8"/>
     </x:row>
     <x:row r="41" ht="20" customHeight="1">
       <x:c r="A41" s="8"/>
@@ -1220,11 +1330,13 @@
       <x:c r="L41" s="9"/>
       <x:c r="M41" s="9"/>
       <x:c r="N41" s="9"/>
-      <x:c r="O41" s="8"/>
-      <x:c r="P41" s="8"/>
+      <x:c r="O41" s="9"/>
+      <x:c r="P41" s="9"/>
       <x:c r="Q41" s="8"/>
       <x:c r="R41" s="8"/>
       <x:c r="S41" s="8"/>
+      <x:c r="T41" s="8"/>
+      <x:c r="U41" s="8"/>
     </x:row>
     <x:row r="42" ht="20" customHeight="1">
       <x:c r="A42" s="8"/>
@@ -1241,11 +1353,13 @@
       <x:c r="L42" s="9"/>
       <x:c r="M42" s="9"/>
       <x:c r="N42" s="9"/>
-      <x:c r="O42" s="8"/>
-      <x:c r="P42" s="8"/>
+      <x:c r="O42" s="9"/>
+      <x:c r="P42" s="9"/>
       <x:c r="Q42" s="8"/>
       <x:c r="R42" s="8"/>
       <x:c r="S42" s="8"/>
+      <x:c r="T42" s="8"/>
+      <x:c r="U42" s="8"/>
     </x:row>
     <x:row r="43" ht="20" customHeight="1">
       <x:c r="A43" s="8"/>
@@ -1262,11 +1376,13 @@
       <x:c r="L43" s="9"/>
       <x:c r="M43" s="9"/>
       <x:c r="N43" s="9"/>
-      <x:c r="O43" s="8"/>
-      <x:c r="P43" s="8"/>
+      <x:c r="O43" s="9"/>
+      <x:c r="P43" s="9"/>
       <x:c r="Q43" s="8"/>
       <x:c r="R43" s="8"/>
       <x:c r="S43" s="8"/>
+      <x:c r="T43" s="8"/>
+      <x:c r="U43" s="8"/>
     </x:row>
     <x:row r="44" ht="20" customHeight="1">
       <x:c r="A44" s="8"/>
@@ -1283,11 +1399,13 @@
       <x:c r="L44" s="9"/>
       <x:c r="M44" s="9"/>
       <x:c r="N44" s="9"/>
-      <x:c r="O44" s="8"/>
-      <x:c r="P44" s="8"/>
+      <x:c r="O44" s="9"/>
+      <x:c r="P44" s="9"/>
       <x:c r="Q44" s="8"/>
       <x:c r="R44" s="8"/>
       <x:c r="S44" s="8"/>
+      <x:c r="T44" s="8"/>
+      <x:c r="U44" s="8"/>
     </x:row>
     <x:row r="45" ht="20" customHeight="1">
       <x:c r="A45" s="8"/>
@@ -1304,11 +1422,13 @@
       <x:c r="L45" s="9"/>
       <x:c r="M45" s="9"/>
       <x:c r="N45" s="9"/>
-      <x:c r="O45" s="8"/>
-      <x:c r="P45" s="8"/>
+      <x:c r="O45" s="9"/>
+      <x:c r="P45" s="9"/>
       <x:c r="Q45" s="8"/>
       <x:c r="R45" s="8"/>
       <x:c r="S45" s="8"/>
+      <x:c r="T45" s="8"/>
+      <x:c r="U45" s="8"/>
     </x:row>
     <x:row r="46" ht="20" customHeight="1">
       <x:c r="A46" s="8"/>
@@ -1325,11 +1445,13 @@
       <x:c r="L46" s="9"/>
       <x:c r="M46" s="9"/>
       <x:c r="N46" s="9"/>
-      <x:c r="O46" s="8"/>
-      <x:c r="P46" s="8"/>
+      <x:c r="O46" s="9"/>
+      <x:c r="P46" s="9"/>
       <x:c r="Q46" s="8"/>
       <x:c r="R46" s="8"/>
       <x:c r="S46" s="8"/>
+      <x:c r="T46" s="8"/>
+      <x:c r="U46" s="8"/>
     </x:row>
     <x:row r="47" ht="20" customHeight="1">
       <x:c r="A47" s="8"/>
@@ -1346,11 +1468,13 @@
       <x:c r="L47" s="9"/>
       <x:c r="M47" s="9"/>
       <x:c r="N47" s="9"/>
-      <x:c r="O47" s="8"/>
-      <x:c r="P47" s="8"/>
+      <x:c r="O47" s="9"/>
+      <x:c r="P47" s="9"/>
       <x:c r="Q47" s="8"/>
       <x:c r="R47" s="8"/>
       <x:c r="S47" s="8"/>
+      <x:c r="T47" s="8"/>
+      <x:c r="U47" s="8"/>
     </x:row>
     <x:row r="48" ht="20" customHeight="1">
       <x:c r="A48" s="8"/>
@@ -1367,11 +1491,13 @@
       <x:c r="L48" s="9"/>
       <x:c r="M48" s="9"/>
       <x:c r="N48" s="9"/>
-      <x:c r="O48" s="8"/>
-      <x:c r="P48" s="8"/>
+      <x:c r="O48" s="9"/>
+      <x:c r="P48" s="9"/>
       <x:c r="Q48" s="8"/>
       <x:c r="R48" s="8"/>
       <x:c r="S48" s="8"/>
+      <x:c r="T48" s="8"/>
+      <x:c r="U48" s="8"/>
     </x:row>
     <x:row r="49" ht="20" customHeight="1">
       <x:c r="A49" s="8"/>
@@ -1388,11 +1514,13 @@
       <x:c r="L49" s="9"/>
       <x:c r="M49" s="9"/>
       <x:c r="N49" s="9"/>
-      <x:c r="O49" s="8"/>
-      <x:c r="P49" s="8"/>
+      <x:c r="O49" s="9"/>
+      <x:c r="P49" s="9"/>
       <x:c r="Q49" s="8"/>
       <x:c r="R49" s="8"/>
       <x:c r="S49" s="8"/>
+      <x:c r="T49" s="8"/>
+      <x:c r="U49" s="8"/>
     </x:row>
     <x:row r="50" ht="20" customHeight="1">
       <x:c r="A50" s="8"/>
@@ -1409,11 +1537,13 @@
       <x:c r="L50" s="9"/>
       <x:c r="M50" s="9"/>
       <x:c r="N50" s="9"/>
-      <x:c r="O50" s="8"/>
-      <x:c r="P50" s="8"/>
+      <x:c r="O50" s="9"/>
+      <x:c r="P50" s="9"/>
       <x:c r="Q50" s="8"/>
       <x:c r="R50" s="8"/>
       <x:c r="S50" s="8"/>
+      <x:c r="T50" s="8"/>
+      <x:c r="U50" s="8"/>
     </x:row>
     <x:row r="51" ht="20" customHeight="1">
       <x:c r="A51" s="8"/>
@@ -1430,11 +1560,13 @@
       <x:c r="L51" s="9"/>
       <x:c r="M51" s="9"/>
       <x:c r="N51" s="9"/>
-      <x:c r="O51" s="8"/>
-      <x:c r="P51" s="8"/>
+      <x:c r="O51" s="9"/>
+      <x:c r="P51" s="9"/>
       <x:c r="Q51" s="8"/>
       <x:c r="R51" s="8"/>
       <x:c r="S51" s="8"/>
+      <x:c r="T51" s="8"/>
+      <x:c r="U51" s="8"/>
     </x:row>
     <x:row r="52" ht="20" customHeight="1">
       <x:c r="A52" s="8"/>
@@ -1451,11 +1583,13 @@
       <x:c r="L52" s="9"/>
       <x:c r="M52" s="9"/>
       <x:c r="N52" s="9"/>
-      <x:c r="O52" s="8"/>
-      <x:c r="P52" s="8"/>
+      <x:c r="O52" s="9"/>
+      <x:c r="P52" s="9"/>
       <x:c r="Q52" s="8"/>
       <x:c r="R52" s="8"/>
       <x:c r="S52" s="8"/>
+      <x:c r="T52" s="8"/>
+      <x:c r="U52" s="8"/>
     </x:row>
     <x:row r="53" ht="20" customHeight="1">
       <x:c r="A53" s="8"/>
@@ -1472,11 +1606,13 @@
       <x:c r="L53" s="9"/>
       <x:c r="M53" s="9"/>
       <x:c r="N53" s="9"/>
-      <x:c r="O53" s="8"/>
-      <x:c r="P53" s="8"/>
+      <x:c r="O53" s="9"/>
+      <x:c r="P53" s="9"/>
       <x:c r="Q53" s="8"/>
       <x:c r="R53" s="8"/>
       <x:c r="S53" s="8"/>
+      <x:c r="T53" s="8"/>
+      <x:c r="U53" s="8"/>
     </x:row>
     <x:row r="54" ht="20" customHeight="1">
       <x:c r="A54" s="8"/>
@@ -1493,11 +1629,13 @@
       <x:c r="L54" s="9"/>
       <x:c r="M54" s="9"/>
       <x:c r="N54" s="9"/>
-      <x:c r="O54" s="8"/>
-      <x:c r="P54" s="8"/>
+      <x:c r="O54" s="9"/>
+      <x:c r="P54" s="9"/>
       <x:c r="Q54" s="8"/>
       <x:c r="R54" s="8"/>
       <x:c r="S54" s="8"/>
+      <x:c r="T54" s="8"/>
+      <x:c r="U54" s="8"/>
     </x:row>
     <x:row r="55" ht="20" customHeight="1">
       <x:c r="A55" s="8"/>
@@ -1514,11 +1652,13 @@
       <x:c r="L55" s="9"/>
       <x:c r="M55" s="9"/>
       <x:c r="N55" s="9"/>
-      <x:c r="O55" s="8"/>
-      <x:c r="P55" s="8"/>
+      <x:c r="O55" s="9"/>
+      <x:c r="P55" s="9"/>
       <x:c r="Q55" s="8"/>
       <x:c r="R55" s="8"/>
       <x:c r="S55" s="8"/>
+      <x:c r="T55" s="8"/>
+      <x:c r="U55" s="8"/>
     </x:row>
     <x:row r="56" ht="20" customHeight="1">
       <x:c r="A56" s="8"/>
@@ -1535,11 +1675,13 @@
       <x:c r="L56" s="9"/>
       <x:c r="M56" s="9"/>
       <x:c r="N56" s="9"/>
-      <x:c r="O56" s="8"/>
-      <x:c r="P56" s="8"/>
+      <x:c r="O56" s="9"/>
+      <x:c r="P56" s="9"/>
       <x:c r="Q56" s="8"/>
       <x:c r="R56" s="8"/>
       <x:c r="S56" s="8"/>
+      <x:c r="T56" s="8"/>
+      <x:c r="U56" s="8"/>
     </x:row>
     <x:row r="57" ht="20" customHeight="1">
       <x:c r="A57" s="8"/>
@@ -1556,11 +1698,13 @@
       <x:c r="L57" s="9"/>
       <x:c r="M57" s="9"/>
       <x:c r="N57" s="9"/>
-      <x:c r="O57" s="8"/>
-      <x:c r="P57" s="8"/>
+      <x:c r="O57" s="9"/>
+      <x:c r="P57" s="9"/>
       <x:c r="Q57" s="8"/>
       <x:c r="R57" s="8"/>
       <x:c r="S57" s="8"/>
+      <x:c r="T57" s="8"/>
+      <x:c r="U57" s="8"/>
     </x:row>
     <x:row r="58" ht="20" customHeight="1">
       <x:c r="A58" s="8"/>
@@ -1577,11 +1721,13 @@
       <x:c r="L58" s="9"/>
       <x:c r="M58" s="9"/>
       <x:c r="N58" s="9"/>
-      <x:c r="O58" s="8"/>
-      <x:c r="P58" s="8"/>
+      <x:c r="O58" s="9"/>
+      <x:c r="P58" s="9"/>
       <x:c r="Q58" s="8"/>
       <x:c r="R58" s="8"/>
       <x:c r="S58" s="8"/>
+      <x:c r="T58" s="8"/>
+      <x:c r="U58" s="8"/>
     </x:row>
     <x:row r="59" ht="20" customHeight="1">
       <x:c r="A59" s="8"/>
@@ -1598,11 +1744,13 @@
       <x:c r="L59" s="9"/>
       <x:c r="M59" s="9"/>
       <x:c r="N59" s="9"/>
-      <x:c r="O59" s="8"/>
-      <x:c r="P59" s="8"/>
+      <x:c r="O59" s="9"/>
+      <x:c r="P59" s="9"/>
       <x:c r="Q59" s="8"/>
       <x:c r="R59" s="8"/>
       <x:c r="S59" s="8"/>
+      <x:c r="T59" s="8"/>
+      <x:c r="U59" s="8"/>
     </x:row>
     <x:row r="60" ht="20" customHeight="1">
       <x:c r="A60" s="8"/>
@@ -1619,11 +1767,13 @@
       <x:c r="L60" s="9"/>
       <x:c r="M60" s="9"/>
       <x:c r="N60" s="9"/>
-      <x:c r="O60" s="8"/>
-      <x:c r="P60" s="8"/>
+      <x:c r="O60" s="9"/>
+      <x:c r="P60" s="9"/>
       <x:c r="Q60" s="8"/>
       <x:c r="R60" s="8"/>
       <x:c r="S60" s="8"/>
+      <x:c r="T60" s="8"/>
+      <x:c r="U60" s="8"/>
     </x:row>
     <x:row r="61" ht="20" customHeight="1">
       <x:c r="A61" s="8"/>
@@ -1640,11 +1790,13 @@
       <x:c r="L61" s="9"/>
       <x:c r="M61" s="9"/>
       <x:c r="N61" s="9"/>
-      <x:c r="O61" s="8"/>
-      <x:c r="P61" s="8"/>
+      <x:c r="O61" s="9"/>
+      <x:c r="P61" s="9"/>
       <x:c r="Q61" s="8"/>
       <x:c r="R61" s="8"/>
       <x:c r="S61" s="8"/>
+      <x:c r="T61" s="8"/>
+      <x:c r="U61" s="8"/>
     </x:row>
     <x:row r="62" ht="20" customHeight="1">
       <x:c r="A62" s="8"/>
@@ -1661,11 +1813,13 @@
       <x:c r="L62" s="9"/>
       <x:c r="M62" s="9"/>
       <x:c r="N62" s="9"/>
-      <x:c r="O62" s="8"/>
-      <x:c r="P62" s="8"/>
+      <x:c r="O62" s="9"/>
+      <x:c r="P62" s="9"/>
       <x:c r="Q62" s="8"/>
       <x:c r="R62" s="8"/>
       <x:c r="S62" s="8"/>
+      <x:c r="T62" s="8"/>
+      <x:c r="U62" s="8"/>
     </x:row>
     <x:row r="63" ht="20" customHeight="1">
       <x:c r="A63" s="8"/>
@@ -1682,11 +1836,13 @@
       <x:c r="L63" s="9"/>
       <x:c r="M63" s="9"/>
       <x:c r="N63" s="9"/>
-      <x:c r="O63" s="8"/>
-      <x:c r="P63" s="8"/>
+      <x:c r="O63" s="9"/>
+      <x:c r="P63" s="9"/>
       <x:c r="Q63" s="8"/>
       <x:c r="R63" s="8"/>
       <x:c r="S63" s="8"/>
+      <x:c r="T63" s="8"/>
+      <x:c r="U63" s="8"/>
     </x:row>
     <x:row r="64" ht="20" customHeight="1">
       <x:c r="A64" s="8"/>
@@ -1703,11 +1859,13 @@
       <x:c r="L64" s="9"/>
       <x:c r="M64" s="9"/>
       <x:c r="N64" s="9"/>
-      <x:c r="O64" s="8"/>
-      <x:c r="P64" s="8"/>
+      <x:c r="O64" s="9"/>
+      <x:c r="P64" s="9"/>
       <x:c r="Q64" s="8"/>
       <x:c r="R64" s="8"/>
       <x:c r="S64" s="8"/>
+      <x:c r="T64" s="8"/>
+      <x:c r="U64" s="8"/>
     </x:row>
     <x:row r="65" ht="20" customHeight="1">
       <x:c r="A65" s="8"/>
@@ -1724,11 +1882,13 @@
       <x:c r="L65" s="9"/>
       <x:c r="M65" s="9"/>
       <x:c r="N65" s="9"/>
-      <x:c r="O65" s="8"/>
-      <x:c r="P65" s="8"/>
+      <x:c r="O65" s="9"/>
+      <x:c r="P65" s="9"/>
       <x:c r="Q65" s="8"/>
       <x:c r="R65" s="8"/>
       <x:c r="S65" s="8"/>
+      <x:c r="T65" s="8"/>
+      <x:c r="U65" s="8"/>
     </x:row>
     <x:row r="66" ht="20" customHeight="1">
       <x:c r="A66" s="8"/>
@@ -1745,11 +1905,13 @@
       <x:c r="L66" s="9"/>
       <x:c r="M66" s="9"/>
       <x:c r="N66" s="9"/>
-      <x:c r="O66" s="8"/>
-      <x:c r="P66" s="8"/>
+      <x:c r="O66" s="9"/>
+      <x:c r="P66" s="9"/>
       <x:c r="Q66" s="8"/>
       <x:c r="R66" s="8"/>
       <x:c r="S66" s="8"/>
+      <x:c r="T66" s="8"/>
+      <x:c r="U66" s="8"/>
     </x:row>
     <x:row r="67" ht="20" customHeight="1">
       <x:c r="A67" s="8"/>
@@ -1766,11 +1928,13 @@
       <x:c r="L67" s="9"/>
       <x:c r="M67" s="9"/>
       <x:c r="N67" s="9"/>
-      <x:c r="O67" s="8"/>
-      <x:c r="P67" s="8"/>
+      <x:c r="O67" s="9"/>
+      <x:c r="P67" s="9"/>
       <x:c r="Q67" s="8"/>
       <x:c r="R67" s="8"/>
       <x:c r="S67" s="8"/>
+      <x:c r="T67" s="8"/>
+      <x:c r="U67" s="8"/>
     </x:row>
     <x:row r="68" ht="20" customHeight="1">
       <x:c r="A68" s="8"/>
@@ -1787,11 +1951,13 @@
       <x:c r="L68" s="9"/>
       <x:c r="M68" s="9"/>
       <x:c r="N68" s="9"/>
-      <x:c r="O68" s="8"/>
-      <x:c r="P68" s="8"/>
+      <x:c r="O68" s="9"/>
+      <x:c r="P68" s="9"/>
       <x:c r="Q68" s="8"/>
       <x:c r="R68" s="8"/>
       <x:c r="S68" s="8"/>
+      <x:c r="T68" s="8"/>
+      <x:c r="U68" s="8"/>
     </x:row>
     <x:row r="69" ht="20" customHeight="1">
       <x:c r="A69" s="8"/>
@@ -1808,11 +1974,13 @@
       <x:c r="L69" s="9"/>
       <x:c r="M69" s="9"/>
       <x:c r="N69" s="9"/>
-      <x:c r="O69" s="8"/>
-      <x:c r="P69" s="8"/>
+      <x:c r="O69" s="9"/>
+      <x:c r="P69" s="9"/>
       <x:c r="Q69" s="8"/>
       <x:c r="R69" s="8"/>
       <x:c r="S69" s="8"/>
+      <x:c r="T69" s="8"/>
+      <x:c r="U69" s="8"/>
     </x:row>
     <x:row r="70" ht="20" customHeight="1">
       <x:c r="A70" s="8"/>
@@ -1829,11 +1997,13 @@
       <x:c r="L70" s="9"/>
       <x:c r="M70" s="9"/>
       <x:c r="N70" s="9"/>
-      <x:c r="O70" s="8"/>
-      <x:c r="P70" s="8"/>
+      <x:c r="O70" s="9"/>
+      <x:c r="P70" s="9"/>
       <x:c r="Q70" s="8"/>
       <x:c r="R70" s="8"/>
       <x:c r="S70" s="8"/>
+      <x:c r="T70" s="8"/>
+      <x:c r="U70" s="8"/>
     </x:row>
     <x:row r="71" ht="20" customHeight="1">
       <x:c r="A71" s="8"/>
@@ -1850,11 +2020,13 @@
       <x:c r="L71" s="9"/>
       <x:c r="M71" s="9"/>
       <x:c r="N71" s="9"/>
-      <x:c r="O71" s="8"/>
-      <x:c r="P71" s="8"/>
+      <x:c r="O71" s="9"/>
+      <x:c r="P71" s="9"/>
       <x:c r="Q71" s="8"/>
       <x:c r="R71" s="8"/>
       <x:c r="S71" s="8"/>
+      <x:c r="T71" s="8"/>
+      <x:c r="U71" s="8"/>
     </x:row>
     <x:row r="72" ht="20" customHeight="1">
       <x:c r="A72" s="8"/>
@@ -1871,11 +2043,13 @@
       <x:c r="L72" s="9"/>
       <x:c r="M72" s="9"/>
       <x:c r="N72" s="9"/>
-      <x:c r="O72" s="8"/>
-      <x:c r="P72" s="8"/>
+      <x:c r="O72" s="9"/>
+      <x:c r="P72" s="9"/>
       <x:c r="Q72" s="8"/>
       <x:c r="R72" s="8"/>
       <x:c r="S72" s="8"/>
+      <x:c r="T72" s="8"/>
+      <x:c r="U72" s="8"/>
     </x:row>
     <x:row r="73" ht="20" customHeight="1">
       <x:c r="A73" s="8"/>
@@ -1892,11 +2066,13 @@
       <x:c r="L73" s="9"/>
       <x:c r="M73" s="9"/>
       <x:c r="N73" s="9"/>
-      <x:c r="O73" s="8"/>
-      <x:c r="P73" s="8"/>
+      <x:c r="O73" s="9"/>
+      <x:c r="P73" s="9"/>
       <x:c r="Q73" s="8"/>
       <x:c r="R73" s="8"/>
       <x:c r="S73" s="8"/>
+      <x:c r="T73" s="8"/>
+      <x:c r="U73" s="8"/>
     </x:row>
     <x:row r="74" ht="20" customHeight="1">
       <x:c r="A74" s="8"/>
@@ -1913,11 +2089,13 @@
       <x:c r="L74" s="9"/>
       <x:c r="M74" s="9"/>
       <x:c r="N74" s="9"/>
-      <x:c r="O74" s="8"/>
-      <x:c r="P74" s="8"/>
+      <x:c r="O74" s="9"/>
+      <x:c r="P74" s="9"/>
       <x:c r="Q74" s="8"/>
       <x:c r="R74" s="8"/>
       <x:c r="S74" s="8"/>
+      <x:c r="T74" s="8"/>
+      <x:c r="U74" s="8"/>
     </x:row>
     <x:row r="75" ht="20" customHeight="1">
       <x:c r="A75" s="8"/>
@@ -1934,11 +2112,13 @@
       <x:c r="L75" s="9"/>
       <x:c r="M75" s="9"/>
       <x:c r="N75" s="9"/>
-      <x:c r="O75" s="8"/>
-      <x:c r="P75" s="8"/>
+      <x:c r="O75" s="9"/>
+      <x:c r="P75" s="9"/>
       <x:c r="Q75" s="8"/>
       <x:c r="R75" s="8"/>
       <x:c r="S75" s="8"/>
+      <x:c r="T75" s="8"/>
+      <x:c r="U75" s="8"/>
     </x:row>
     <x:row r="76" ht="20" customHeight="1">
       <x:c r="A76" s="8"/>
@@ -1955,11 +2135,13 @@
       <x:c r="L76" s="9"/>
       <x:c r="M76" s="9"/>
       <x:c r="N76" s="9"/>
-      <x:c r="O76" s="8"/>
-      <x:c r="P76" s="8"/>
+      <x:c r="O76" s="9"/>
+      <x:c r="P76" s="9"/>
       <x:c r="Q76" s="8"/>
       <x:c r="R76" s="8"/>
       <x:c r="S76" s="8"/>
+      <x:c r="T76" s="8"/>
+      <x:c r="U76" s="8"/>
     </x:row>
     <x:row r="77" ht="20" customHeight="1">
       <x:c r="A77" s="8"/>
@@ -1976,11 +2158,13 @@
       <x:c r="L77" s="9"/>
       <x:c r="M77" s="9"/>
       <x:c r="N77" s="9"/>
-      <x:c r="O77" s="8"/>
-      <x:c r="P77" s="8"/>
+      <x:c r="O77" s="9"/>
+      <x:c r="P77" s="9"/>
       <x:c r="Q77" s="8"/>
       <x:c r="R77" s="8"/>
       <x:c r="S77" s="8"/>
+      <x:c r="T77" s="8"/>
+      <x:c r="U77" s="8"/>
     </x:row>
     <x:row r="78" ht="20" customHeight="1">
       <x:c r="A78" s="8"/>
@@ -1997,11 +2181,13 @@
       <x:c r="L78" s="9"/>
       <x:c r="M78" s="9"/>
       <x:c r="N78" s="9"/>
-      <x:c r="O78" s="8"/>
-      <x:c r="P78" s="8"/>
+      <x:c r="O78" s="9"/>
+      <x:c r="P78" s="9"/>
       <x:c r="Q78" s="8"/>
       <x:c r="R78" s="8"/>
       <x:c r="S78" s="8"/>
+      <x:c r="T78" s="8"/>
+      <x:c r="U78" s="8"/>
     </x:row>
     <x:row r="79" ht="20" customHeight="1">
       <x:c r="A79" s="8"/>
@@ -2018,11 +2204,13 @@
       <x:c r="L79" s="9"/>
       <x:c r="M79" s="9"/>
       <x:c r="N79" s="9"/>
-      <x:c r="O79" s="8"/>
-      <x:c r="P79" s="8"/>
+      <x:c r="O79" s="9"/>
+      <x:c r="P79" s="9"/>
       <x:c r="Q79" s="8"/>
       <x:c r="R79" s="8"/>
       <x:c r="S79" s="8"/>
+      <x:c r="T79" s="8"/>
+      <x:c r="U79" s="8"/>
     </x:row>
     <x:row r="80" ht="20" customHeight="1">
       <x:c r="A80" s="8"/>
@@ -2039,11 +2227,13 @@
       <x:c r="L80" s="9"/>
       <x:c r="M80" s="9"/>
       <x:c r="N80" s="9"/>
-      <x:c r="O80" s="8"/>
-      <x:c r="P80" s="8"/>
+      <x:c r="O80" s="9"/>
+      <x:c r="P80" s="9"/>
       <x:c r="Q80" s="8"/>
       <x:c r="R80" s="8"/>
       <x:c r="S80" s="8"/>
+      <x:c r="T80" s="8"/>
+      <x:c r="U80" s="8"/>
     </x:row>
     <x:row r="81" ht="20" customHeight="1">
       <x:c r="A81" s="8"/>
@@ -2060,11 +2250,13 @@
       <x:c r="L81" s="9"/>
       <x:c r="M81" s="9"/>
       <x:c r="N81" s="9"/>
-      <x:c r="O81" s="8"/>
-      <x:c r="P81" s="8"/>
+      <x:c r="O81" s="9"/>
+      <x:c r="P81" s="9"/>
       <x:c r="Q81" s="8"/>
       <x:c r="R81" s="8"/>
       <x:c r="S81" s="8"/>
+      <x:c r="T81" s="8"/>
+      <x:c r="U81" s="8"/>
     </x:row>
     <x:row r="82" ht="20" customHeight="1">
       <x:c r="A82" s="8"/>
@@ -2081,11 +2273,13 @@
       <x:c r="L82" s="9"/>
       <x:c r="M82" s="9"/>
       <x:c r="N82" s="9"/>
-      <x:c r="O82" s="8"/>
-      <x:c r="P82" s="8"/>
+      <x:c r="O82" s="9"/>
+      <x:c r="P82" s="9"/>
       <x:c r="Q82" s="8"/>
       <x:c r="R82" s="8"/>
       <x:c r="S82" s="8"/>
+      <x:c r="T82" s="8"/>
+      <x:c r="U82" s="8"/>
     </x:row>
     <x:row r="83" ht="20" customHeight="1">
       <x:c r="A83" s="8"/>
@@ -2102,11 +2296,13 @@
       <x:c r="L83" s="9"/>
       <x:c r="M83" s="9"/>
       <x:c r="N83" s="9"/>
-      <x:c r="O83" s="8"/>
-      <x:c r="P83" s="8"/>
+      <x:c r="O83" s="9"/>
+      <x:c r="P83" s="9"/>
       <x:c r="Q83" s="8"/>
       <x:c r="R83" s="8"/>
       <x:c r="S83" s="8"/>
+      <x:c r="T83" s="8"/>
+      <x:c r="U83" s="8"/>
     </x:row>
     <x:row r="84" ht="20" customHeight="1">
       <x:c r="A84" s="8"/>
@@ -2123,11 +2319,13 @@
       <x:c r="L84" s="9"/>
       <x:c r="M84" s="9"/>
       <x:c r="N84" s="9"/>
-      <x:c r="O84" s="8"/>
-      <x:c r="P84" s="8"/>
+      <x:c r="O84" s="9"/>
+      <x:c r="P84" s="9"/>
       <x:c r="Q84" s="8"/>
       <x:c r="R84" s="8"/>
       <x:c r="S84" s="8"/>
+      <x:c r="T84" s="8"/>
+      <x:c r="U84" s="8"/>
     </x:row>
     <x:row r="85" ht="20" customHeight="1">
       <x:c r="A85" s="8"/>
@@ -2144,11 +2342,13 @@
       <x:c r="L85" s="9"/>
       <x:c r="M85" s="9"/>
       <x:c r="N85" s="9"/>
-      <x:c r="O85" s="8"/>
-      <x:c r="P85" s="8"/>
+      <x:c r="O85" s="9"/>
+      <x:c r="P85" s="9"/>
       <x:c r="Q85" s="8"/>
       <x:c r="R85" s="8"/>
       <x:c r="S85" s="8"/>
+      <x:c r="T85" s="8"/>
+      <x:c r="U85" s="8"/>
     </x:row>
     <x:row r="86" ht="20" customHeight="1">
       <x:c r="A86" s="8"/>
@@ -2165,11 +2365,13 @@
       <x:c r="L86" s="9"/>
       <x:c r="M86" s="9"/>
       <x:c r="N86" s="9"/>
-      <x:c r="O86" s="8"/>
-      <x:c r="P86" s="8"/>
+      <x:c r="O86" s="9"/>
+      <x:c r="P86" s="9"/>
       <x:c r="Q86" s="8"/>
       <x:c r="R86" s="8"/>
       <x:c r="S86" s="8"/>
+      <x:c r="T86" s="8"/>
+      <x:c r="U86" s="8"/>
     </x:row>
     <x:row r="87" ht="20" customHeight="1">
       <x:c r="A87" s="8"/>
@@ -2186,11 +2388,13 @@
       <x:c r="L87" s="9"/>
       <x:c r="M87" s="9"/>
       <x:c r="N87" s="9"/>
-      <x:c r="O87" s="8"/>
-      <x:c r="P87" s="8"/>
+      <x:c r="O87" s="9"/>
+      <x:c r="P87" s="9"/>
       <x:c r="Q87" s="8"/>
       <x:c r="R87" s="8"/>
       <x:c r="S87" s="8"/>
+      <x:c r="T87" s="8"/>
+      <x:c r="U87" s="8"/>
     </x:row>
     <x:row r="88" ht="20" customHeight="1">
       <x:c r="A88" s="8"/>
@@ -2207,11 +2411,13 @@
       <x:c r="L88" s="9"/>
       <x:c r="M88" s="9"/>
       <x:c r="N88" s="9"/>
-      <x:c r="O88" s="8"/>
-      <x:c r="P88" s="8"/>
+      <x:c r="O88" s="9"/>
+      <x:c r="P88" s="9"/>
       <x:c r="Q88" s="8"/>
       <x:c r="R88" s="8"/>
       <x:c r="S88" s="8"/>
+      <x:c r="T88" s="8"/>
+      <x:c r="U88" s="8"/>
     </x:row>
     <x:row r="89" ht="20" customHeight="1">
       <x:c r="A89" s="8"/>
@@ -2228,11 +2434,13 @@
       <x:c r="L89" s="9"/>
       <x:c r="M89" s="9"/>
       <x:c r="N89" s="9"/>
-      <x:c r="O89" s="8"/>
-      <x:c r="P89" s="8"/>
+      <x:c r="O89" s="9"/>
+      <x:c r="P89" s="9"/>
       <x:c r="Q89" s="8"/>
       <x:c r="R89" s="8"/>
       <x:c r="S89" s="8"/>
+      <x:c r="T89" s="8"/>
+      <x:c r="U89" s="8"/>
     </x:row>
     <x:row r="90" ht="20" customHeight="1">
       <x:c r="A90" s="8"/>
@@ -2249,11 +2457,13 @@
       <x:c r="L90" s="9"/>
       <x:c r="M90" s="9"/>
       <x:c r="N90" s="9"/>
-      <x:c r="O90" s="8"/>
-      <x:c r="P90" s="8"/>
+      <x:c r="O90" s="9"/>
+      <x:c r="P90" s="9"/>
       <x:c r="Q90" s="8"/>
       <x:c r="R90" s="8"/>
       <x:c r="S90" s="8"/>
+      <x:c r="T90" s="8"/>
+      <x:c r="U90" s="8"/>
     </x:row>
     <x:row r="91" ht="20" customHeight="1">
       <x:c r="A91" s="8"/>
@@ -2270,11 +2480,13 @@
       <x:c r="L91" s="9"/>
       <x:c r="M91" s="9"/>
       <x:c r="N91" s="9"/>
-      <x:c r="O91" s="8"/>
-      <x:c r="P91" s="8"/>
+      <x:c r="O91" s="9"/>
+      <x:c r="P91" s="9"/>
       <x:c r="Q91" s="8"/>
       <x:c r="R91" s="8"/>
       <x:c r="S91" s="8"/>
+      <x:c r="T91" s="8"/>
+      <x:c r="U91" s="8"/>
     </x:row>
     <x:row r="92" ht="20" customHeight="1">
       <x:c r="A92" s="8"/>
@@ -2291,11 +2503,13 @@
       <x:c r="L92" s="9"/>
       <x:c r="M92" s="9"/>
       <x:c r="N92" s="9"/>
-      <x:c r="O92" s="8"/>
-      <x:c r="P92" s="8"/>
+      <x:c r="O92" s="9"/>
+      <x:c r="P92" s="9"/>
       <x:c r="Q92" s="8"/>
       <x:c r="R92" s="8"/>
       <x:c r="S92" s="8"/>
+      <x:c r="T92" s="8"/>
+      <x:c r="U92" s="8"/>
     </x:row>
     <x:row r="93" ht="20" customHeight="1">
       <x:c r="A93" s="8"/>
@@ -2312,11 +2526,13 @@
       <x:c r="L93" s="9"/>
       <x:c r="M93" s="9"/>
       <x:c r="N93" s="9"/>
-      <x:c r="O93" s="8"/>
-      <x:c r="P93" s="8"/>
+      <x:c r="O93" s="9"/>
+      <x:c r="P93" s="9"/>
       <x:c r="Q93" s="8"/>
       <x:c r="R93" s="8"/>
       <x:c r="S93" s="8"/>
+      <x:c r="T93" s="8"/>
+      <x:c r="U93" s="8"/>
     </x:row>
     <x:row r="94" ht="20" customHeight="1">
       <x:c r="A94" s="8"/>
@@ -2333,11 +2549,13 @@
       <x:c r="L94" s="9"/>
       <x:c r="M94" s="9"/>
       <x:c r="N94" s="9"/>
-      <x:c r="O94" s="8"/>
-      <x:c r="P94" s="8"/>
+      <x:c r="O94" s="9"/>
+      <x:c r="P94" s="9"/>
       <x:c r="Q94" s="8"/>
       <x:c r="R94" s="8"/>
       <x:c r="S94" s="8"/>
+      <x:c r="T94" s="8"/>
+      <x:c r="U94" s="8"/>
     </x:row>
     <x:row r="95" ht="20" customHeight="1">
       <x:c r="A95" s="8"/>
@@ -2354,11 +2572,13 @@
       <x:c r="L95" s="9"/>
       <x:c r="M95" s="9"/>
       <x:c r="N95" s="9"/>
-      <x:c r="O95" s="8"/>
-      <x:c r="P95" s="8"/>
+      <x:c r="O95" s="9"/>
+      <x:c r="P95" s="9"/>
       <x:c r="Q95" s="8"/>
       <x:c r="R95" s="8"/>
       <x:c r="S95" s="8"/>
+      <x:c r="T95" s="8"/>
+      <x:c r="U95" s="8"/>
     </x:row>
     <x:row r="96" ht="20" customHeight="1">
       <x:c r="A96" s="8"/>
@@ -2375,11 +2595,13 @@
       <x:c r="L96" s="9"/>
       <x:c r="M96" s="9"/>
       <x:c r="N96" s="9"/>
-      <x:c r="O96" s="8"/>
-      <x:c r="P96" s="8"/>
+      <x:c r="O96" s="9"/>
+      <x:c r="P96" s="9"/>
       <x:c r="Q96" s="8"/>
       <x:c r="R96" s="8"/>
       <x:c r="S96" s="8"/>
+      <x:c r="T96" s="8"/>
+      <x:c r="U96" s="8"/>
     </x:row>
     <x:row r="97" ht="20" customHeight="1">
       <x:c r="A97" s="8"/>
@@ -2396,11 +2618,13 @@
       <x:c r="L97" s="9"/>
       <x:c r="M97" s="9"/>
       <x:c r="N97" s="9"/>
-      <x:c r="O97" s="8"/>
-      <x:c r="P97" s="8"/>
+      <x:c r="O97" s="9"/>
+      <x:c r="P97" s="9"/>
       <x:c r="Q97" s="8"/>
       <x:c r="R97" s="8"/>
       <x:c r="S97" s="8"/>
+      <x:c r="T97" s="8"/>
+      <x:c r="U97" s="8"/>
     </x:row>
     <x:row r="98" ht="20" customHeight="1">
       <x:c r="A98" s="8"/>
@@ -2417,11 +2641,13 @@
       <x:c r="L98" s="9"/>
       <x:c r="M98" s="9"/>
       <x:c r="N98" s="9"/>
-      <x:c r="O98" s="8"/>
-      <x:c r="P98" s="8"/>
+      <x:c r="O98" s="9"/>
+      <x:c r="P98" s="9"/>
       <x:c r="Q98" s="8"/>
       <x:c r="R98" s="8"/>
       <x:c r="S98" s="8"/>
+      <x:c r="T98" s="8"/>
+      <x:c r="U98" s="8"/>
     </x:row>
     <x:row r="99" ht="20" customHeight="1">
       <x:c r="A99" s="8"/>
@@ -2438,11 +2664,13 @@
       <x:c r="L99" s="9"/>
       <x:c r="M99" s="9"/>
       <x:c r="N99" s="9"/>
-      <x:c r="O99" s="8"/>
-      <x:c r="P99" s="8"/>
+      <x:c r="O99" s="9"/>
+      <x:c r="P99" s="9"/>
       <x:c r="Q99" s="8"/>
       <x:c r="R99" s="8"/>
       <x:c r="S99" s="8"/>
+      <x:c r="T99" s="8"/>
+      <x:c r="U99" s="8"/>
     </x:row>
     <x:row r="100" ht="20" customHeight="1">
       <x:c r="A100" s="8"/>
@@ -2459,11 +2687,13 @@
       <x:c r="L100" s="9"/>
       <x:c r="M100" s="9"/>
       <x:c r="N100" s="9"/>
-      <x:c r="O100" s="8"/>
-      <x:c r="P100" s="8"/>
+      <x:c r="O100" s="9"/>
+      <x:c r="P100" s="9"/>
       <x:c r="Q100" s="8"/>
       <x:c r="R100" s="8"/>
       <x:c r="S100" s="8"/>
+      <x:c r="T100" s="8"/>
+      <x:c r="U100" s="8"/>
     </x:row>
     <x:row r="101" ht="20" customHeight="1">
       <x:c r="A101" s="8"/>
@@ -2480,11 +2710,13 @@
       <x:c r="L101" s="9"/>
       <x:c r="M101" s="9"/>
       <x:c r="N101" s="9"/>
-      <x:c r="O101" s="8"/>
-      <x:c r="P101" s="8"/>
+      <x:c r="O101" s="9"/>
+      <x:c r="P101" s="9"/>
       <x:c r="Q101" s="8"/>
       <x:c r="R101" s="8"/>
       <x:c r="S101" s="8"/>
+      <x:c r="T101" s="8"/>
+      <x:c r="U101" s="8"/>
     </x:row>
     <x:row r="102" ht="20" customHeight="1">
       <x:c r="A102" s="8"/>
@@ -2501,11 +2733,13 @@
       <x:c r="L102" s="9"/>
       <x:c r="M102" s="9"/>
       <x:c r="N102" s="9"/>
-      <x:c r="O102" s="8"/>
-      <x:c r="P102" s="8"/>
+      <x:c r="O102" s="9"/>
+      <x:c r="P102" s="9"/>
       <x:c r="Q102" s="8"/>
       <x:c r="R102" s="8"/>
       <x:c r="S102" s="8"/>
+      <x:c r="T102" s="8"/>
+      <x:c r="U102" s="8"/>
     </x:row>
     <x:row r="103" ht="20" customHeight="1">
       <x:c r="A103" s="8"/>
@@ -2522,11 +2756,13 @@
       <x:c r="L103" s="9"/>
       <x:c r="M103" s="9"/>
       <x:c r="N103" s="9"/>
-      <x:c r="O103" s="8"/>
-      <x:c r="P103" s="8"/>
+      <x:c r="O103" s="9"/>
+      <x:c r="P103" s="9"/>
       <x:c r="Q103" s="8"/>
       <x:c r="R103" s="8"/>
       <x:c r="S103" s="8"/>
+      <x:c r="T103" s="8"/>
+      <x:c r="U103" s="8"/>
     </x:row>
     <x:row r="104" ht="20" customHeight="1">
       <x:c r="A104" s="8"/>
@@ -2543,11 +2779,13 @@
       <x:c r="L104" s="9"/>
       <x:c r="M104" s="9"/>
       <x:c r="N104" s="9"/>
-      <x:c r="O104" s="8"/>
-      <x:c r="P104" s="8"/>
+      <x:c r="O104" s="9"/>
+      <x:c r="P104" s="9"/>
       <x:c r="Q104" s="8"/>
       <x:c r="R104" s="8"/>
       <x:c r="S104" s="8"/>
+      <x:c r="T104" s="8"/>
+      <x:c r="U104" s="8"/>
     </x:row>
     <x:row r="105" ht="20" customHeight="1">
       <x:c r="A105" s="8"/>
@@ -2564,11 +2802,13 @@
       <x:c r="L105" s="9"/>
       <x:c r="M105" s="9"/>
       <x:c r="N105" s="9"/>
-      <x:c r="O105" s="8"/>
-      <x:c r="P105" s="8"/>
+      <x:c r="O105" s="9"/>
+      <x:c r="P105" s="9"/>
       <x:c r="Q105" s="8"/>
       <x:c r="R105" s="8"/>
       <x:c r="S105" s="8"/>
+      <x:c r="T105" s="8"/>
+      <x:c r="U105" s="8"/>
     </x:row>
     <x:row r="106" ht="20" customHeight="1">
       <x:c r="A106" s="8"/>
@@ -2585,11 +2825,13 @@
       <x:c r="L106" s="9"/>
       <x:c r="M106" s="9"/>
       <x:c r="N106" s="9"/>
-      <x:c r="O106" s="8"/>
-      <x:c r="P106" s="8"/>
+      <x:c r="O106" s="9"/>
+      <x:c r="P106" s="9"/>
       <x:c r="Q106" s="8"/>
       <x:c r="R106" s="8"/>
       <x:c r="S106" s="8"/>
+      <x:c r="T106" s="8"/>
+      <x:c r="U106" s="8"/>
     </x:row>
     <x:row r="107" ht="20" customHeight="1">
       <x:c r="A107" s="8"/>
@@ -2606,11 +2848,13 @@
       <x:c r="L107" s="9"/>
       <x:c r="M107" s="9"/>
       <x:c r="N107" s="9"/>
-      <x:c r="O107" s="8"/>
-      <x:c r="P107" s="8"/>
+      <x:c r="O107" s="9"/>
+      <x:c r="P107" s="9"/>
       <x:c r="Q107" s="8"/>
       <x:c r="R107" s="8"/>
       <x:c r="S107" s="8"/>
+      <x:c r="T107" s="8"/>
+      <x:c r="U107" s="8"/>
     </x:row>
     <x:row r="108" ht="20" customHeight="1">
       <x:c r="A108" s="8"/>
@@ -2627,11 +2871,13 @@
       <x:c r="L108" s="9"/>
       <x:c r="M108" s="9"/>
       <x:c r="N108" s="9"/>
-      <x:c r="O108" s="8"/>
-      <x:c r="P108" s="8"/>
+      <x:c r="O108" s="9"/>
+      <x:c r="P108" s="9"/>
       <x:c r="Q108" s="8"/>
       <x:c r="R108" s="8"/>
       <x:c r="S108" s="8"/>
+      <x:c r="T108" s="8"/>
+      <x:c r="U108" s="8"/>
     </x:row>
     <x:row r="109" ht="20" customHeight="1">
       <x:c r="A109" s="8"/>
@@ -2648,11 +2894,13 @@
       <x:c r="L109" s="9"/>
       <x:c r="M109" s="9"/>
       <x:c r="N109" s="9"/>
-      <x:c r="O109" s="8"/>
-      <x:c r="P109" s="8"/>
+      <x:c r="O109" s="9"/>
+      <x:c r="P109" s="9"/>
       <x:c r="Q109" s="8"/>
       <x:c r="R109" s="8"/>
       <x:c r="S109" s="8"/>
+      <x:c r="T109" s="8"/>
+      <x:c r="U109" s="8"/>
     </x:row>
     <x:row r="110" ht="20" customHeight="1">
       <x:c r="A110" s="8"/>
@@ -2669,11 +2917,13 @@
       <x:c r="L110" s="9"/>
       <x:c r="M110" s="9"/>
       <x:c r="N110" s="9"/>
-      <x:c r="O110" s="8"/>
-      <x:c r="P110" s="8"/>
+      <x:c r="O110" s="9"/>
+      <x:c r="P110" s="9"/>
       <x:c r="Q110" s="8"/>
       <x:c r="R110" s="8"/>
       <x:c r="S110" s="8"/>
+      <x:c r="T110" s="8"/>
+      <x:c r="U110" s="8"/>
     </x:row>
     <x:row r="111" ht="20" customHeight="1">
       <x:c r="A111" s="8"/>
@@ -2690,11 +2940,13 @@
       <x:c r="L111" s="9"/>
       <x:c r="M111" s="9"/>
       <x:c r="N111" s="9"/>
-      <x:c r="O111" s="8"/>
-      <x:c r="P111" s="8"/>
+      <x:c r="O111" s="9"/>
+      <x:c r="P111" s="9"/>
       <x:c r="Q111" s="8"/>
       <x:c r="R111" s="8"/>
       <x:c r="S111" s="8"/>
+      <x:c r="T111" s="8"/>
+      <x:c r="U111" s="8"/>
     </x:row>
     <x:row r="112" ht="20" customHeight="1">
       <x:c r="A112" s="8"/>
@@ -2711,11 +2963,13 @@
       <x:c r="L112" s="9"/>
       <x:c r="M112" s="9"/>
       <x:c r="N112" s="9"/>
-      <x:c r="O112" s="8"/>
-      <x:c r="P112" s="8"/>
+      <x:c r="O112" s="9"/>
+      <x:c r="P112" s="9"/>
       <x:c r="Q112" s="8"/>
       <x:c r="R112" s="8"/>
       <x:c r="S112" s="8"/>
+      <x:c r="T112" s="8"/>
+      <x:c r="U112" s="8"/>
     </x:row>
     <x:row r="113" ht="20" customHeight="1">
       <x:c r="A113" s="8"/>
@@ -2732,11 +2986,13 @@
       <x:c r="L113" s="9"/>
       <x:c r="M113" s="9"/>
       <x:c r="N113" s="9"/>
-      <x:c r="O113" s="8"/>
-      <x:c r="P113" s="8"/>
+      <x:c r="O113" s="9"/>
+      <x:c r="P113" s="9"/>
       <x:c r="Q113" s="8"/>
       <x:c r="R113" s="8"/>
       <x:c r="S113" s="8"/>
+      <x:c r="T113" s="8"/>
+      <x:c r="U113" s="8"/>
     </x:row>
     <x:row r="114" ht="20" customHeight="1">
       <x:c r="A114" s="8"/>
@@ -2753,11 +3009,13 @@
       <x:c r="L114" s="9"/>
       <x:c r="M114" s="9"/>
       <x:c r="N114" s="9"/>
-      <x:c r="O114" s="8"/>
-      <x:c r="P114" s="8"/>
+      <x:c r="O114" s="9"/>
+      <x:c r="P114" s="9"/>
       <x:c r="Q114" s="8"/>
       <x:c r="R114" s="8"/>
       <x:c r="S114" s="8"/>
+      <x:c r="T114" s="8"/>
+      <x:c r="U114" s="8"/>
     </x:row>
     <x:row r="115" ht="20" customHeight="1">
       <x:c r="A115" s="8"/>
@@ -2774,11 +3032,13 @@
       <x:c r="L115" s="9"/>
       <x:c r="M115" s="9"/>
       <x:c r="N115" s="9"/>
-      <x:c r="O115" s="8"/>
-      <x:c r="P115" s="8"/>
+      <x:c r="O115" s="9"/>
+      <x:c r="P115" s="9"/>
       <x:c r="Q115" s="8"/>
       <x:c r="R115" s="8"/>
       <x:c r="S115" s="8"/>
+      <x:c r="T115" s="8"/>
+      <x:c r="U115" s="8"/>
     </x:row>
     <x:row r="116" ht="20" customHeight="1">
       <x:c r="A116" s="8"/>
@@ -2795,11 +3055,13 @@
       <x:c r="L116" s="9"/>
       <x:c r="M116" s="9"/>
       <x:c r="N116" s="9"/>
-      <x:c r="O116" s="8"/>
-      <x:c r="P116" s="8"/>
+      <x:c r="O116" s="9"/>
+      <x:c r="P116" s="9"/>
       <x:c r="Q116" s="8"/>
       <x:c r="R116" s="8"/>
       <x:c r="S116" s="8"/>
+      <x:c r="T116" s="8"/>
+      <x:c r="U116" s="8"/>
     </x:row>
     <x:row r="117" ht="20" customHeight="1">
       <x:c r="A117" s="8"/>
@@ -2816,11 +3078,13 @@
       <x:c r="L117" s="9"/>
       <x:c r="M117" s="9"/>
       <x:c r="N117" s="9"/>
-      <x:c r="O117" s="8"/>
-      <x:c r="P117" s="8"/>
+      <x:c r="O117" s="9"/>
+      <x:c r="P117" s="9"/>
       <x:c r="Q117" s="8"/>
       <x:c r="R117" s="8"/>
       <x:c r="S117" s="8"/>
+      <x:c r="T117" s="8"/>
+      <x:c r="U117" s="8"/>
     </x:row>
     <x:row r="118" ht="20" customHeight="1">
       <x:c r="A118" s="8"/>
@@ -2837,11 +3101,13 @@
       <x:c r="L118" s="9"/>
       <x:c r="M118" s="9"/>
       <x:c r="N118" s="9"/>
-      <x:c r="O118" s="8"/>
-      <x:c r="P118" s="8"/>
+      <x:c r="O118" s="9"/>
+      <x:c r="P118" s="9"/>
       <x:c r="Q118" s="8"/>
       <x:c r="R118" s="8"/>
       <x:c r="S118" s="8"/>
+      <x:c r="T118" s="8"/>
+      <x:c r="U118" s="8"/>
     </x:row>
     <x:row r="119" ht="20" customHeight="1">
       <x:c r="A119" s="8"/>
@@ -2858,11 +3124,13 @@
       <x:c r="L119" s="9"/>
       <x:c r="M119" s="9"/>
       <x:c r="N119" s="9"/>
-      <x:c r="O119" s="8"/>
-      <x:c r="P119" s="8"/>
+      <x:c r="O119" s="9"/>
+      <x:c r="P119" s="9"/>
       <x:c r="Q119" s="8"/>
       <x:c r="R119" s="8"/>
       <x:c r="S119" s="8"/>
+      <x:c r="T119" s="8"/>
+      <x:c r="U119" s="8"/>
     </x:row>
     <x:row r="120" ht="20" customHeight="1">
       <x:c r="A120" s="8"/>
@@ -2879,11 +3147,13 @@
       <x:c r="L120" s="9"/>
       <x:c r="M120" s="9"/>
       <x:c r="N120" s="9"/>
-      <x:c r="O120" s="8"/>
-      <x:c r="P120" s="8"/>
+      <x:c r="O120" s="9"/>
+      <x:c r="P120" s="9"/>
       <x:c r="Q120" s="8"/>
       <x:c r="R120" s="8"/>
       <x:c r="S120" s="8"/>
+      <x:c r="T120" s="8"/>
+      <x:c r="U120" s="8"/>
     </x:row>
     <x:row r="121" ht="20" customHeight="1">
       <x:c r="A121" s="8"/>
@@ -2900,11 +3170,13 @@
       <x:c r="L121" s="9"/>
       <x:c r="M121" s="9"/>
       <x:c r="N121" s="9"/>
-      <x:c r="O121" s="8"/>
-      <x:c r="P121" s="8"/>
+      <x:c r="O121" s="9"/>
+      <x:c r="P121" s="9"/>
       <x:c r="Q121" s="8"/>
       <x:c r="R121" s="8"/>
       <x:c r="S121" s="8"/>
+      <x:c r="T121" s="8"/>
+      <x:c r="U121" s="8"/>
     </x:row>
     <x:row r="122" ht="20" customHeight="1">
       <x:c r="A122" s="8"/>
@@ -2921,11 +3193,13 @@
       <x:c r="L122" s="9"/>
       <x:c r="M122" s="9"/>
       <x:c r="N122" s="9"/>
-      <x:c r="O122" s="8"/>
-      <x:c r="P122" s="8"/>
+      <x:c r="O122" s="9"/>
+      <x:c r="P122" s="9"/>
       <x:c r="Q122" s="8"/>
       <x:c r="R122" s="8"/>
       <x:c r="S122" s="8"/>
+      <x:c r="T122" s="8"/>
+      <x:c r="U122" s="8"/>
     </x:row>
     <x:row r="123" ht="20" customHeight="1">
       <x:c r="A123" s="8"/>
@@ -2942,11 +3216,13 @@
       <x:c r="L123" s="9"/>
       <x:c r="M123" s="9"/>
       <x:c r="N123" s="9"/>
-      <x:c r="O123" s="8"/>
-      <x:c r="P123" s="8"/>
+      <x:c r="O123" s="9"/>
+      <x:c r="P123" s="9"/>
       <x:c r="Q123" s="8"/>
       <x:c r="R123" s="8"/>
       <x:c r="S123" s="8"/>
+      <x:c r="T123" s="8"/>
+      <x:c r="U123" s="8"/>
     </x:row>
     <x:row r="124" ht="20" customHeight="1">
       <x:c r="A124" s="8"/>
@@ -2963,11 +3239,13 @@
       <x:c r="L124" s="9"/>
       <x:c r="M124" s="9"/>
       <x:c r="N124" s="9"/>
-      <x:c r="O124" s="8"/>
-      <x:c r="P124" s="8"/>
+      <x:c r="O124" s="9"/>
+      <x:c r="P124" s="9"/>
       <x:c r="Q124" s="8"/>
       <x:c r="R124" s="8"/>
       <x:c r="S124" s="8"/>
+      <x:c r="T124" s="8"/>
+      <x:c r="U124" s="8"/>
     </x:row>
     <x:row r="125" ht="20" customHeight="1">
       <x:c r="A125" s="8"/>
@@ -2984,11 +3262,13 @@
       <x:c r="L125" s="9"/>
       <x:c r="M125" s="9"/>
       <x:c r="N125" s="9"/>
-      <x:c r="O125" s="8"/>
-      <x:c r="P125" s="8"/>
+      <x:c r="O125" s="9"/>
+      <x:c r="P125" s="9"/>
       <x:c r="Q125" s="8"/>
       <x:c r="R125" s="8"/>
       <x:c r="S125" s="8"/>
+      <x:c r="T125" s="8"/>
+      <x:c r="U125" s="8"/>
     </x:row>
     <x:row r="126" ht="20" customHeight="1">
       <x:c r="A126" s="8"/>
@@ -3005,11 +3285,13 @@
       <x:c r="L126" s="9"/>
       <x:c r="M126" s="9"/>
       <x:c r="N126" s="9"/>
-      <x:c r="O126" s="8"/>
-      <x:c r="P126" s="8"/>
+      <x:c r="O126" s="9"/>
+      <x:c r="P126" s="9"/>
       <x:c r="Q126" s="8"/>
       <x:c r="R126" s="8"/>
       <x:c r="S126" s="8"/>
+      <x:c r="T126" s="8"/>
+      <x:c r="U126" s="8"/>
     </x:row>
     <x:row r="127" ht="20" customHeight="1">
       <x:c r="A127" s="8"/>
@@ -3026,11 +3308,13 @@
       <x:c r="L127" s="9"/>
       <x:c r="M127" s="9"/>
       <x:c r="N127" s="9"/>
-      <x:c r="O127" s="8"/>
-      <x:c r="P127" s="8"/>
+      <x:c r="O127" s="9"/>
+      <x:c r="P127" s="9"/>
       <x:c r="Q127" s="8"/>
       <x:c r="R127" s="8"/>
       <x:c r="S127" s="8"/>
+      <x:c r="T127" s="8"/>
+      <x:c r="U127" s="8"/>
     </x:row>
     <x:row r="128" ht="20" customHeight="1">
       <x:c r="A128" s="8"/>
@@ -3047,11 +3331,13 @@
       <x:c r="L128" s="9"/>
       <x:c r="M128" s="9"/>
       <x:c r="N128" s="9"/>
-      <x:c r="O128" s="8"/>
-      <x:c r="P128" s="8"/>
+      <x:c r="O128" s="9"/>
+      <x:c r="P128" s="9"/>
       <x:c r="Q128" s="8"/>
       <x:c r="R128" s="8"/>
       <x:c r="S128" s="8"/>
+      <x:c r="T128" s="8"/>
+      <x:c r="U128" s="8"/>
     </x:row>
     <x:row r="129" ht="20" customHeight="1">
       <x:c r="A129" s="8"/>
@@ -3068,11 +3354,13 @@
       <x:c r="L129" s="9"/>
       <x:c r="M129" s="9"/>
       <x:c r="N129" s="9"/>
-      <x:c r="O129" s="8"/>
-      <x:c r="P129" s="8"/>
+      <x:c r="O129" s="9"/>
+      <x:c r="P129" s="9"/>
       <x:c r="Q129" s="8"/>
       <x:c r="R129" s="8"/>
       <x:c r="S129" s="8"/>
+      <x:c r="T129" s="8"/>
+      <x:c r="U129" s="8"/>
     </x:row>
     <x:row r="130" ht="20" customHeight="1">
       <x:c r="A130" s="8"/>
@@ -3089,11 +3377,13 @@
       <x:c r="L130" s="9"/>
       <x:c r="M130" s="9"/>
       <x:c r="N130" s="9"/>
-      <x:c r="O130" s="8"/>
-      <x:c r="P130" s="8"/>
+      <x:c r="O130" s="9"/>
+      <x:c r="P130" s="9"/>
       <x:c r="Q130" s="8"/>
       <x:c r="R130" s="8"/>
       <x:c r="S130" s="8"/>
+      <x:c r="T130" s="8"/>
+      <x:c r="U130" s="8"/>
     </x:row>
     <x:row r="131" ht="20" customHeight="1">
       <x:c r="A131" s="8"/>
@@ -3110,11 +3400,13 @@
       <x:c r="L131" s="9"/>
       <x:c r="M131" s="9"/>
       <x:c r="N131" s="9"/>
-      <x:c r="O131" s="8"/>
-      <x:c r="P131" s="8"/>
+      <x:c r="O131" s="9"/>
+      <x:c r="P131" s="9"/>
       <x:c r="Q131" s="8"/>
       <x:c r="R131" s="8"/>
       <x:c r="S131" s="8"/>
+      <x:c r="T131" s="8"/>
+      <x:c r="U131" s="8"/>
     </x:row>
     <x:row r="132" ht="20" customHeight="1">
       <x:c r="A132" s="8"/>
@@ -3131,11 +3423,13 @@
       <x:c r="L132" s="9"/>
       <x:c r="M132" s="9"/>
       <x:c r="N132" s="9"/>
-      <x:c r="O132" s="8"/>
-      <x:c r="P132" s="8"/>
+      <x:c r="O132" s="9"/>
+      <x:c r="P132" s="9"/>
       <x:c r="Q132" s="8"/>
       <x:c r="R132" s="8"/>
       <x:c r="S132" s="8"/>
+      <x:c r="T132" s="8"/>
+      <x:c r="U132" s="8"/>
     </x:row>
     <x:row r="133" ht="20" customHeight="1">
       <x:c r="A133" s="8"/>
@@ -3152,11 +3446,13 @@
       <x:c r="L133" s="9"/>
       <x:c r="M133" s="9"/>
       <x:c r="N133" s="9"/>
-      <x:c r="O133" s="8"/>
-      <x:c r="P133" s="8"/>
+      <x:c r="O133" s="9"/>
+      <x:c r="P133" s="9"/>
       <x:c r="Q133" s="8"/>
       <x:c r="R133" s="8"/>
       <x:c r="S133" s="8"/>
+      <x:c r="T133" s="8"/>
+      <x:c r="U133" s="8"/>
     </x:row>
     <x:row r="134" ht="20" customHeight="1">
       <x:c r="A134" s="8"/>
@@ -3173,11 +3469,13 @@
       <x:c r="L134" s="9"/>
       <x:c r="M134" s="9"/>
       <x:c r="N134" s="9"/>
-      <x:c r="O134" s="8"/>
-      <x:c r="P134" s="8"/>
+      <x:c r="O134" s="9"/>
+      <x:c r="P134" s="9"/>
       <x:c r="Q134" s="8"/>
       <x:c r="R134" s="8"/>
       <x:c r="S134" s="8"/>
+      <x:c r="T134" s="8"/>
+      <x:c r="U134" s="8"/>
     </x:row>
     <x:row r="135" ht="20" customHeight="1">
       <x:c r="A135" s="8"/>
@@ -3194,11 +3492,13 @@
       <x:c r="L135" s="9"/>
       <x:c r="M135" s="9"/>
       <x:c r="N135" s="9"/>
-      <x:c r="O135" s="8"/>
-      <x:c r="P135" s="8"/>
+      <x:c r="O135" s="9"/>
+      <x:c r="P135" s="9"/>
       <x:c r="Q135" s="8"/>
       <x:c r="R135" s="8"/>
       <x:c r="S135" s="8"/>
+      <x:c r="T135" s="8"/>
+      <x:c r="U135" s="8"/>
     </x:row>
     <x:row r="136" ht="20" customHeight="1">
       <x:c r="A136" s="8"/>
@@ -3215,11 +3515,13 @@
       <x:c r="L136" s="9"/>
       <x:c r="M136" s="9"/>
       <x:c r="N136" s="9"/>
-      <x:c r="O136" s="8"/>
-      <x:c r="P136" s="8"/>
+      <x:c r="O136" s="9"/>
+      <x:c r="P136" s="9"/>
       <x:c r="Q136" s="8"/>
       <x:c r="R136" s="8"/>
       <x:c r="S136" s="8"/>
+      <x:c r="T136" s="8"/>
+      <x:c r="U136" s="8"/>
     </x:row>
     <x:row r="137" ht="20" customHeight="1">
       <x:c r="A137" s="8"/>
@@ -3236,11 +3538,13 @@
       <x:c r="L137" s="9"/>
       <x:c r="M137" s="9"/>
       <x:c r="N137" s="9"/>
-      <x:c r="O137" s="8"/>
-      <x:c r="P137" s="8"/>
+      <x:c r="O137" s="9"/>
+      <x:c r="P137" s="9"/>
       <x:c r="Q137" s="8"/>
       <x:c r="R137" s="8"/>
       <x:c r="S137" s="8"/>
+      <x:c r="T137" s="8"/>
+      <x:c r="U137" s="8"/>
     </x:row>
     <x:row r="138" ht="20" customHeight="1">
       <x:c r="A138" s="8"/>
@@ -3257,11 +3561,13 @@
       <x:c r="L138" s="9"/>
       <x:c r="M138" s="9"/>
       <x:c r="N138" s="9"/>
-      <x:c r="O138" s="8"/>
-      <x:c r="P138" s="8"/>
+      <x:c r="O138" s="9"/>
+      <x:c r="P138" s="9"/>
       <x:c r="Q138" s="8"/>
       <x:c r="R138" s="8"/>
       <x:c r="S138" s="8"/>
+      <x:c r="T138" s="8"/>
+      <x:c r="U138" s="8"/>
     </x:row>
     <x:row r="139" ht="20" customHeight="1">
       <x:c r="A139" s="8"/>
@@ -3278,11 +3584,13 @@
       <x:c r="L139" s="9"/>
       <x:c r="M139" s="9"/>
       <x:c r="N139" s="9"/>
-      <x:c r="O139" s="8"/>
-      <x:c r="P139" s="8"/>
+      <x:c r="O139" s="9"/>
+      <x:c r="P139" s="9"/>
       <x:c r="Q139" s="8"/>
       <x:c r="R139" s="8"/>
       <x:c r="S139" s="8"/>
+      <x:c r="T139" s="8"/>
+      <x:c r="U139" s="8"/>
     </x:row>
     <x:row r="140" ht="20" customHeight="1">
       <x:c r="A140" s="8"/>
@@ -3299,11 +3607,13 @@
       <x:c r="L140" s="9"/>
       <x:c r="M140" s="9"/>
       <x:c r="N140" s="9"/>
-      <x:c r="O140" s="8"/>
-      <x:c r="P140" s="8"/>
+      <x:c r="O140" s="9"/>
+      <x:c r="P140" s="9"/>
       <x:c r="Q140" s="8"/>
       <x:c r="R140" s="8"/>
       <x:c r="S140" s="8"/>
+      <x:c r="T140" s="8"/>
+      <x:c r="U140" s="8"/>
     </x:row>
     <x:row r="141" ht="20" customHeight="1">
       <x:c r="A141" s="8"/>
@@ -3320,11 +3630,13 @@
       <x:c r="L141" s="9"/>
       <x:c r="M141" s="9"/>
       <x:c r="N141" s="9"/>
-      <x:c r="O141" s="8"/>
-      <x:c r="P141" s="8"/>
+      <x:c r="O141" s="9"/>
+      <x:c r="P141" s="9"/>
       <x:c r="Q141" s="8"/>
       <x:c r="R141" s="8"/>
       <x:c r="S141" s="8"/>
+      <x:c r="T141" s="8"/>
+      <x:c r="U141" s="8"/>
     </x:row>
     <x:row r="142" ht="20" customHeight="1">
       <x:c r="A142" s="8"/>
@@ -3341,11 +3653,13 @@
       <x:c r="L142" s="9"/>
       <x:c r="M142" s="9"/>
       <x:c r="N142" s="9"/>
-      <x:c r="O142" s="8"/>
-      <x:c r="P142" s="8"/>
+      <x:c r="O142" s="9"/>
+      <x:c r="P142" s="9"/>
       <x:c r="Q142" s="8"/>
       <x:c r="R142" s="8"/>
       <x:c r="S142" s="8"/>
+      <x:c r="T142" s="8"/>
+      <x:c r="U142" s="8"/>
     </x:row>
     <x:row r="143" ht="20" customHeight="1">
       <x:c r="A143" s="8"/>
@@ -3362,11 +3676,13 @@
       <x:c r="L143" s="9"/>
       <x:c r="M143" s="9"/>
       <x:c r="N143" s="9"/>
-      <x:c r="O143" s="8"/>
-      <x:c r="P143" s="8"/>
+      <x:c r="O143" s="9"/>
+      <x:c r="P143" s="9"/>
       <x:c r="Q143" s="8"/>
       <x:c r="R143" s="8"/>
       <x:c r="S143" s="8"/>
+      <x:c r="T143" s="8"/>
+      <x:c r="U143" s="8"/>
     </x:row>
     <x:row r="144" ht="20" customHeight="1">
       <x:c r="A144" s="8"/>
@@ -3383,11 +3699,13 @@
       <x:c r="L144" s="9"/>
       <x:c r="M144" s="9"/>
       <x:c r="N144" s="9"/>
-      <x:c r="O144" s="8"/>
-      <x:c r="P144" s="8"/>
+      <x:c r="O144" s="9"/>
+      <x:c r="P144" s="9"/>
       <x:c r="Q144" s="8"/>
       <x:c r="R144" s="8"/>
       <x:c r="S144" s="8"/>
+      <x:c r="T144" s="8"/>
+      <x:c r="U144" s="8"/>
     </x:row>
     <x:row r="145" ht="20" customHeight="1">
       <x:c r="A145" s="8"/>
@@ -3404,11 +3722,13 @@
       <x:c r="L145" s="9"/>
       <x:c r="M145" s="9"/>
       <x:c r="N145" s="9"/>
-      <x:c r="O145" s="8"/>
-      <x:c r="P145" s="8"/>
+      <x:c r="O145" s="9"/>
+      <x:c r="P145" s="9"/>
       <x:c r="Q145" s="8"/>
       <x:c r="R145" s="8"/>
       <x:c r="S145" s="8"/>
+      <x:c r="T145" s="8"/>
+      <x:c r="U145" s="8"/>
     </x:row>
     <x:row r="146" ht="20" customHeight="1">
       <x:c r="A146" s="8"/>
@@ -3425,11 +3745,13 @@
       <x:c r="L146" s="9"/>
       <x:c r="M146" s="9"/>
       <x:c r="N146" s="9"/>
-      <x:c r="O146" s="8"/>
-      <x:c r="P146" s="8"/>
+      <x:c r="O146" s="9"/>
+      <x:c r="P146" s="9"/>
       <x:c r="Q146" s="8"/>
       <x:c r="R146" s="8"/>
       <x:c r="S146" s="8"/>
+      <x:c r="T146" s="8"/>
+      <x:c r="U146" s="8"/>
     </x:row>
     <x:row r="147" ht="20" customHeight="1">
       <x:c r="A147" s="8"/>
@@ -3446,11 +3768,13 @@
       <x:c r="L147" s="9"/>
       <x:c r="M147" s="9"/>
       <x:c r="N147" s="9"/>
-      <x:c r="O147" s="8"/>
-      <x:c r="P147" s="8"/>
+      <x:c r="O147" s="9"/>
+      <x:c r="P147" s="9"/>
       <x:c r="Q147" s="8"/>
       <x:c r="R147" s="8"/>
       <x:c r="S147" s="8"/>
+      <x:c r="T147" s="8"/>
+      <x:c r="U147" s="8"/>
     </x:row>
     <x:row r="148" ht="20" customHeight="1">
       <x:c r="A148" s="8"/>
@@ -3467,11 +3791,13 @@
       <x:c r="L148" s="9"/>
       <x:c r="M148" s="9"/>
       <x:c r="N148" s="9"/>
-      <x:c r="O148" s="8"/>
-      <x:c r="P148" s="8"/>
+      <x:c r="O148" s="9"/>
+      <x:c r="P148" s="9"/>
       <x:c r="Q148" s="8"/>
       <x:c r="R148" s="8"/>
       <x:c r="S148" s="8"/>
+      <x:c r="T148" s="8"/>
+      <x:c r="U148" s="8"/>
     </x:row>
     <x:row r="149" ht="20" customHeight="1">
       <x:c r="A149" s="8"/>
@@ -3488,11 +3814,13 @@
       <x:c r="L149" s="9"/>
       <x:c r="M149" s="9"/>
       <x:c r="N149" s="9"/>
-      <x:c r="O149" s="8"/>
-      <x:c r="P149" s="8"/>
+      <x:c r="O149" s="9"/>
+      <x:c r="P149" s="9"/>
       <x:c r="Q149" s="8"/>
       <x:c r="R149" s="8"/>
       <x:c r="S149" s="8"/>
+      <x:c r="T149" s="8"/>
+      <x:c r="U149" s="8"/>
     </x:row>
     <x:row r="150" ht="20" customHeight="1">
       <x:c r="A150" s="8"/>
@@ -3509,11 +3837,13 @@
       <x:c r="L150" s="9"/>
       <x:c r="M150" s="9"/>
       <x:c r="N150" s="9"/>
-      <x:c r="O150" s="8"/>
-      <x:c r="P150" s="8"/>
+      <x:c r="O150" s="9"/>
+      <x:c r="P150" s="9"/>
       <x:c r="Q150" s="8"/>
       <x:c r="R150" s="8"/>
       <x:c r="S150" s="8"/>
+      <x:c r="T150" s="8"/>
+      <x:c r="U150" s="8"/>
     </x:row>
     <x:row r="151" ht="20" customHeight="1">
       <x:c r="A151" s="8"/>
@@ -3530,11 +3860,13 @@
       <x:c r="L151" s="9"/>
       <x:c r="M151" s="9"/>
       <x:c r="N151" s="9"/>
-      <x:c r="O151" s="8"/>
-      <x:c r="P151" s="8"/>
+      <x:c r="O151" s="9"/>
+      <x:c r="P151" s="9"/>
       <x:c r="Q151" s="8"/>
       <x:c r="R151" s="8"/>
       <x:c r="S151" s="8"/>
+      <x:c r="T151" s="8"/>
+      <x:c r="U151" s="8"/>
     </x:row>
     <x:row r="152" ht="20" customHeight="1">
       <x:c r="A152" s="8"/>
@@ -3551,11 +3883,13 @@
       <x:c r="L152" s="9"/>
       <x:c r="M152" s="9"/>
       <x:c r="N152" s="9"/>
-      <x:c r="O152" s="8"/>
-      <x:c r="P152" s="8"/>
+      <x:c r="O152" s="9"/>
+      <x:c r="P152" s="9"/>
       <x:c r="Q152" s="8"/>
       <x:c r="R152" s="8"/>
       <x:c r="S152" s="8"/>
+      <x:c r="T152" s="8"/>
+      <x:c r="U152" s="8"/>
     </x:row>
     <x:row r="153" ht="20" customHeight="1">
       <x:c r="A153" s="8"/>
@@ -3572,11 +3906,13 @@
       <x:c r="L153" s="9"/>
       <x:c r="M153" s="9"/>
       <x:c r="N153" s="9"/>
-      <x:c r="O153" s="8"/>
-      <x:c r="P153" s="8"/>
+      <x:c r="O153" s="9"/>
+      <x:c r="P153" s="9"/>
       <x:c r="Q153" s="8"/>
       <x:c r="R153" s="8"/>
       <x:c r="S153" s="8"/>
+      <x:c r="T153" s="8"/>
+      <x:c r="U153" s="8"/>
     </x:row>
     <x:row r="154" ht="20" customHeight="1">
       <x:c r="A154" s="8"/>
@@ -3593,11 +3929,13 @@
       <x:c r="L154" s="9"/>
       <x:c r="M154" s="9"/>
       <x:c r="N154" s="9"/>
-      <x:c r="O154" s="8"/>
-      <x:c r="P154" s="8"/>
+      <x:c r="O154" s="9"/>
+      <x:c r="P154" s="9"/>
       <x:c r="Q154" s="8"/>
       <x:c r="R154" s="8"/>
       <x:c r="S154" s="8"/>
+      <x:c r="T154" s="8"/>
+      <x:c r="U154" s="8"/>
     </x:row>
     <x:row r="155" ht="20" customHeight="1">
       <x:c r="A155" s="8"/>
@@ -3614,11 +3952,13 @@
       <x:c r="L155" s="9"/>
       <x:c r="M155" s="9"/>
       <x:c r="N155" s="9"/>
-      <x:c r="O155" s="8"/>
-      <x:c r="P155" s="8"/>
+      <x:c r="O155" s="9"/>
+      <x:c r="P155" s="9"/>
       <x:c r="Q155" s="8"/>
       <x:c r="R155" s="8"/>
       <x:c r="S155" s="8"/>
+      <x:c r="T155" s="8"/>
+      <x:c r="U155" s="8"/>
     </x:row>
     <x:row r="156" ht="20" customHeight="1">
       <x:c r="A156" s="8"/>
@@ -3635,11 +3975,13 @@
       <x:c r="L156" s="9"/>
       <x:c r="M156" s="9"/>
       <x:c r="N156" s="9"/>
-      <x:c r="O156" s="8"/>
-      <x:c r="P156" s="8"/>
+      <x:c r="O156" s="9"/>
+      <x:c r="P156" s="9"/>
       <x:c r="Q156" s="8"/>
       <x:c r="R156" s="8"/>
       <x:c r="S156" s="8"/>
+      <x:c r="T156" s="8"/>
+      <x:c r="U156" s="8"/>
     </x:row>
     <x:row r="157" ht="20" customHeight="1">
       <x:c r="A157" s="8"/>
@@ -3656,11 +3998,13 @@
       <x:c r="L157" s="9"/>
       <x:c r="M157" s="9"/>
       <x:c r="N157" s="9"/>
-      <x:c r="O157" s="8"/>
-      <x:c r="P157" s="8"/>
+      <x:c r="O157" s="9"/>
+      <x:c r="P157" s="9"/>
       <x:c r="Q157" s="8"/>
       <x:c r="R157" s="8"/>
       <x:c r="S157" s="8"/>
+      <x:c r="T157" s="8"/>
+      <x:c r="U157" s="8"/>
     </x:row>
     <x:row r="158" ht="20" customHeight="1">
       <x:c r="A158" s="8"/>
@@ -3677,11 +4021,13 @@
       <x:c r="L158" s="9"/>
       <x:c r="M158" s="9"/>
       <x:c r="N158" s="9"/>
-      <x:c r="O158" s="8"/>
-      <x:c r="P158" s="8"/>
+      <x:c r="O158" s="9"/>
+      <x:c r="P158" s="9"/>
       <x:c r="Q158" s="8"/>
       <x:c r="R158" s="8"/>
       <x:c r="S158" s="8"/>
+      <x:c r="T158" s="8"/>
+      <x:c r="U158" s="8"/>
     </x:row>
     <x:row r="159" ht="20" customHeight="1">
       <x:c r="A159" s="8"/>
@@ -3698,11 +4044,13 @@
       <x:c r="L159" s="9"/>
       <x:c r="M159" s="9"/>
       <x:c r="N159" s="9"/>
-      <x:c r="O159" s="8"/>
-      <x:c r="P159" s="8"/>
+      <x:c r="O159" s="9"/>
+      <x:c r="P159" s="9"/>
       <x:c r="Q159" s="8"/>
       <x:c r="R159" s="8"/>
       <x:c r="S159" s="8"/>
+      <x:c r="T159" s="8"/>
+      <x:c r="U159" s="8"/>
     </x:row>
     <x:row r="160" ht="20" customHeight="1">
       <x:c r="A160" s="8"/>
@@ -3719,11 +4067,13 @@
       <x:c r="L160" s="9"/>
       <x:c r="M160" s="9"/>
       <x:c r="N160" s="9"/>
-      <x:c r="O160" s="8"/>
-      <x:c r="P160" s="8"/>
+      <x:c r="O160" s="9"/>
+      <x:c r="P160" s="9"/>
       <x:c r="Q160" s="8"/>
       <x:c r="R160" s="8"/>
       <x:c r="S160" s="8"/>
+      <x:c r="T160" s="8"/>
+      <x:c r="U160" s="8"/>
     </x:row>
     <x:row r="161" ht="20" customHeight="1">
       <x:c r="A161" s="8"/>
@@ -3740,11 +4090,13 @@
       <x:c r="L161" s="9"/>
       <x:c r="M161" s="9"/>
       <x:c r="N161" s="9"/>
-      <x:c r="O161" s="8"/>
-      <x:c r="P161" s="8"/>
+      <x:c r="O161" s="9"/>
+      <x:c r="P161" s="9"/>
       <x:c r="Q161" s="8"/>
       <x:c r="R161" s="8"/>
       <x:c r="S161" s="8"/>
+      <x:c r="T161" s="8"/>
+      <x:c r="U161" s="8"/>
     </x:row>
     <x:row r="162" ht="20" customHeight="1">
       <x:c r="A162" s="8"/>
@@ -3761,11 +4113,13 @@
       <x:c r="L162" s="9"/>
       <x:c r="M162" s="9"/>
       <x:c r="N162" s="9"/>
-      <x:c r="O162" s="8"/>
-      <x:c r="P162" s="8"/>
+      <x:c r="O162" s="9"/>
+      <x:c r="P162" s="9"/>
       <x:c r="Q162" s="8"/>
       <x:c r="R162" s="8"/>
       <x:c r="S162" s="8"/>
+      <x:c r="T162" s="8"/>
+      <x:c r="U162" s="8"/>
     </x:row>
     <x:row r="163" ht="20" customHeight="1">
       <x:c r="A163" s="8"/>
@@ -3782,11 +4136,13 @@
       <x:c r="L163" s="9"/>
       <x:c r="M163" s="9"/>
       <x:c r="N163" s="9"/>
-      <x:c r="O163" s="8"/>
-      <x:c r="P163" s="8"/>
+      <x:c r="O163" s="9"/>
+      <x:c r="P163" s="9"/>
       <x:c r="Q163" s="8"/>
       <x:c r="R163" s="8"/>
       <x:c r="S163" s="8"/>
+      <x:c r="T163" s="8"/>
+      <x:c r="U163" s="8"/>
     </x:row>
     <x:row r="164" ht="20" customHeight="1">
       <x:c r="A164" s="8"/>
@@ -3803,11 +4159,13 @@
       <x:c r="L164" s="9"/>
       <x:c r="M164" s="9"/>
       <x:c r="N164" s="9"/>
-      <x:c r="O164" s="8"/>
-      <x:c r="P164" s="8"/>
+      <x:c r="O164" s="9"/>
+      <x:c r="P164" s="9"/>
       <x:c r="Q164" s="8"/>
       <x:c r="R164" s="8"/>
       <x:c r="S164" s="8"/>
+      <x:c r="T164" s="8"/>
+      <x:c r="U164" s="8"/>
     </x:row>
     <x:row r="165" ht="20" customHeight="1">
       <x:c r="A165" s="8"/>
@@ -3824,11 +4182,13 @@
       <x:c r="L165" s="9"/>
       <x:c r="M165" s="9"/>
       <x:c r="N165" s="9"/>
-      <x:c r="O165" s="8"/>
-      <x:c r="P165" s="8"/>
+      <x:c r="O165" s="9"/>
+      <x:c r="P165" s="9"/>
       <x:c r="Q165" s="8"/>
       <x:c r="R165" s="8"/>
       <x:c r="S165" s="8"/>
+      <x:c r="T165" s="8"/>
+      <x:c r="U165" s="8"/>
     </x:row>
     <x:row r="166" ht="20" customHeight="1">
       <x:c r="A166" s="8"/>
@@ -3845,11 +4205,13 @@
       <x:c r="L166" s="9"/>
       <x:c r="M166" s="9"/>
       <x:c r="N166" s="9"/>
-      <x:c r="O166" s="8"/>
-      <x:c r="P166" s="8"/>
+      <x:c r="O166" s="9"/>
+      <x:c r="P166" s="9"/>
       <x:c r="Q166" s="8"/>
       <x:c r="R166" s="8"/>
       <x:c r="S166" s="8"/>
+      <x:c r="T166" s="8"/>
+      <x:c r="U166" s="8"/>
     </x:row>
     <x:row r="167" ht="20" customHeight="1">
       <x:c r="A167" s="8"/>
@@ -3866,11 +4228,13 @@
       <x:c r="L167" s="9"/>
       <x:c r="M167" s="9"/>
       <x:c r="N167" s="9"/>
-      <x:c r="O167" s="8"/>
-      <x:c r="P167" s="8"/>
+      <x:c r="O167" s="9"/>
+      <x:c r="P167" s="9"/>
       <x:c r="Q167" s="8"/>
       <x:c r="R167" s="8"/>
       <x:c r="S167" s="8"/>
+      <x:c r="T167" s="8"/>
+      <x:c r="U167" s="8"/>
     </x:row>
     <x:row r="168" ht="20" customHeight="1">
       <x:c r="A168" s="8"/>
@@ -3887,11 +4251,13 @@
       <x:c r="L168" s="9"/>
       <x:c r="M168" s="9"/>
       <x:c r="N168" s="9"/>
-      <x:c r="O168" s="8"/>
-      <x:c r="P168" s="8"/>
+      <x:c r="O168" s="9"/>
+      <x:c r="P168" s="9"/>
       <x:c r="Q168" s="8"/>
       <x:c r="R168" s="8"/>
       <x:c r="S168" s="8"/>
+      <x:c r="T168" s="8"/>
+      <x:c r="U168" s="8"/>
     </x:row>
     <x:row r="169" ht="20" customHeight="1">
       <x:c r="A169" s="8"/>
@@ -3908,11 +4274,13 @@
       <x:c r="L169" s="9"/>
       <x:c r="M169" s="9"/>
       <x:c r="N169" s="9"/>
-      <x:c r="O169" s="8"/>
-      <x:c r="P169" s="8"/>
+      <x:c r="O169" s="9"/>
+      <x:c r="P169" s="9"/>
       <x:c r="Q169" s="8"/>
       <x:c r="R169" s="8"/>
       <x:c r="S169" s="8"/>
+      <x:c r="T169" s="8"/>
+      <x:c r="U169" s="8"/>
     </x:row>
     <x:row r="170" ht="20" customHeight="1">
       <x:c r="A170" s="8"/>
@@ -3929,11 +4297,13 @@
       <x:c r="L170" s="9"/>
       <x:c r="M170" s="9"/>
       <x:c r="N170" s="9"/>
-      <x:c r="O170" s="8"/>
-      <x:c r="P170" s="8"/>
+      <x:c r="O170" s="9"/>
+      <x:c r="P170" s="9"/>
       <x:c r="Q170" s="8"/>
       <x:c r="R170" s="8"/>
       <x:c r="S170" s="8"/>
+      <x:c r="T170" s="8"/>
+      <x:c r="U170" s="8"/>
     </x:row>
     <x:row r="171" ht="20" customHeight="1">
       <x:c r="A171" s="8"/>
@@ -3950,11 +4320,13 @@
       <x:c r="L171" s="9"/>
       <x:c r="M171" s="9"/>
       <x:c r="N171" s="9"/>
-      <x:c r="O171" s="8"/>
-      <x:c r="P171" s="8"/>
+      <x:c r="O171" s="9"/>
+      <x:c r="P171" s="9"/>
       <x:c r="Q171" s="8"/>
       <x:c r="R171" s="8"/>
       <x:c r="S171" s="8"/>
+      <x:c r="T171" s="8"/>
+      <x:c r="U171" s="8"/>
     </x:row>
     <x:row r="172" ht="20" customHeight="1">
       <x:c r="A172" s="8"/>
@@ -3971,11 +4343,13 @@
       <x:c r="L172" s="9"/>
       <x:c r="M172" s="9"/>
       <x:c r="N172" s="9"/>
-      <x:c r="O172" s="8"/>
-      <x:c r="P172" s="8"/>
+      <x:c r="O172" s="9"/>
+      <x:c r="P172" s="9"/>
       <x:c r="Q172" s="8"/>
       <x:c r="R172" s="8"/>
       <x:c r="S172" s="8"/>
+      <x:c r="T172" s="8"/>
+      <x:c r="U172" s="8"/>
     </x:row>
     <x:row r="173" ht="20" customHeight="1">
       <x:c r="A173" s="8"/>
@@ -3992,11 +4366,13 @@
       <x:c r="L173" s="9"/>
       <x:c r="M173" s="9"/>
       <x:c r="N173" s="9"/>
-      <x:c r="O173" s="8"/>
-      <x:c r="P173" s="8"/>
+      <x:c r="O173" s="9"/>
+      <x:c r="P173" s="9"/>
       <x:c r="Q173" s="8"/>
       <x:c r="R173" s="8"/>
       <x:c r="S173" s="8"/>
+      <x:c r="T173" s="8"/>
+      <x:c r="U173" s="8"/>
     </x:row>
     <x:row r="174" ht="20" customHeight="1">
       <x:c r="A174" s="8"/>
@@ -4013,11 +4389,13 @@
       <x:c r="L174" s="9"/>
       <x:c r="M174" s="9"/>
       <x:c r="N174" s="9"/>
-      <x:c r="O174" s="8"/>
-      <x:c r="P174" s="8"/>
+      <x:c r="O174" s="9"/>
+      <x:c r="P174" s="9"/>
       <x:c r="Q174" s="8"/>
       <x:c r="R174" s="8"/>
       <x:c r="S174" s="8"/>
+      <x:c r="T174" s="8"/>
+      <x:c r="U174" s="8"/>
     </x:row>
     <x:row r="175" ht="20" customHeight="1">
       <x:c r="A175" s="8"/>
@@ -4034,11 +4412,13 @@
       <x:c r="L175" s="9"/>
       <x:c r="M175" s="9"/>
       <x:c r="N175" s="9"/>
-      <x:c r="O175" s="8"/>
-      <x:c r="P175" s="8"/>
+      <x:c r="O175" s="9"/>
+      <x:c r="P175" s="9"/>
       <x:c r="Q175" s="8"/>
       <x:c r="R175" s="8"/>
       <x:c r="S175" s="8"/>
+      <x:c r="T175" s="8"/>
+      <x:c r="U175" s="8"/>
     </x:row>
     <x:row r="176" ht="20" customHeight="1">
       <x:c r="A176" s="8"/>
@@ -4055,11 +4435,13 @@
       <x:c r="L176" s="9"/>
       <x:c r="M176" s="9"/>
       <x:c r="N176" s="9"/>
-      <x:c r="O176" s="8"/>
-      <x:c r="P176" s="8"/>
+      <x:c r="O176" s="9"/>
+      <x:c r="P176" s="9"/>
       <x:c r="Q176" s="8"/>
       <x:c r="R176" s="8"/>
       <x:c r="S176" s="8"/>
+      <x:c r="T176" s="8"/>
+      <x:c r="U176" s="8"/>
     </x:row>
     <x:row r="177" ht="20" customHeight="1">
       <x:c r="A177" s="8"/>
@@ -4076,11 +4458,13 @@
       <x:c r="L177" s="9"/>
       <x:c r="M177" s="9"/>
       <x:c r="N177" s="9"/>
-      <x:c r="O177" s="8"/>
-      <x:c r="P177" s="8"/>
+      <x:c r="O177" s="9"/>
+      <x:c r="P177" s="9"/>
       <x:c r="Q177" s="8"/>
       <x:c r="R177" s="8"/>
       <x:c r="S177" s="8"/>
+      <x:c r="T177" s="8"/>
+      <x:c r="U177" s="8"/>
     </x:row>
     <x:row r="178" ht="20" customHeight="1">
       <x:c r="A178" s="8"/>
@@ -4097,11 +4481,13 @@
       <x:c r="L178" s="9"/>
       <x:c r="M178" s="9"/>
       <x:c r="N178" s="9"/>
-      <x:c r="O178" s="8"/>
-      <x:c r="P178" s="8"/>
+      <x:c r="O178" s="9"/>
+      <x:c r="P178" s="9"/>
       <x:c r="Q178" s="8"/>
       <x:c r="R178" s="8"/>
       <x:c r="S178" s="8"/>
+      <x:c r="T178" s="8"/>
+      <x:c r="U178" s="8"/>
     </x:row>
     <x:row r="179" ht="20" customHeight="1">
       <x:c r="A179" s="8"/>
@@ -4118,11 +4504,13 @@
       <x:c r="L179" s="9"/>
       <x:c r="M179" s="9"/>
       <x:c r="N179" s="9"/>
-      <x:c r="O179" s="8"/>
-      <x:c r="P179" s="8"/>
+      <x:c r="O179" s="9"/>
+      <x:c r="P179" s="9"/>
       <x:c r="Q179" s="8"/>
       <x:c r="R179" s="8"/>
       <x:c r="S179" s="8"/>
+      <x:c r="T179" s="8"/>
+      <x:c r="U179" s="8"/>
     </x:row>
     <x:row r="180" ht="20" customHeight="1">
       <x:c r="A180" s="8"/>
@@ -4139,11 +4527,13 @@
       <x:c r="L180" s="9"/>
       <x:c r="M180" s="9"/>
       <x:c r="N180" s="9"/>
-      <x:c r="O180" s="8"/>
-      <x:c r="P180" s="8"/>
+      <x:c r="O180" s="9"/>
+      <x:c r="P180" s="9"/>
       <x:c r="Q180" s="8"/>
       <x:c r="R180" s="8"/>
       <x:c r="S180" s="8"/>
+      <x:c r="T180" s="8"/>
+      <x:c r="U180" s="8"/>
     </x:row>
     <x:row r="181" ht="20" customHeight="1">
       <x:c r="A181" s="8"/>
@@ -4160,11 +4550,13 @@
       <x:c r="L181" s="9"/>
       <x:c r="M181" s="9"/>
       <x:c r="N181" s="9"/>
-      <x:c r="O181" s="8"/>
-      <x:c r="P181" s="8"/>
+      <x:c r="O181" s="9"/>
+      <x:c r="P181" s="9"/>
       <x:c r="Q181" s="8"/>
       <x:c r="R181" s="8"/>
       <x:c r="S181" s="8"/>
+      <x:c r="T181" s="8"/>
+      <x:c r="U181" s="8"/>
     </x:row>
     <x:row r="182" ht="20" customHeight="1">
       <x:c r="A182" s="8"/>
@@ -4181,11 +4573,13 @@
       <x:c r="L182" s="9"/>
       <x:c r="M182" s="9"/>
       <x:c r="N182" s="9"/>
-      <x:c r="O182" s="8"/>
-      <x:c r="P182" s="8"/>
+      <x:c r="O182" s="9"/>
+      <x:c r="P182" s="9"/>
       <x:c r="Q182" s="8"/>
       <x:c r="R182" s="8"/>
       <x:c r="S182" s="8"/>
+      <x:c r="T182" s="8"/>
+      <x:c r="U182" s="8"/>
     </x:row>
     <x:row r="183" ht="20" customHeight="1">
       <x:c r="A183" s="8"/>
@@ -4202,11 +4596,13 @@
       <x:c r="L183" s="9"/>
       <x:c r="M183" s="9"/>
       <x:c r="N183" s="9"/>
-      <x:c r="O183" s="8"/>
-      <x:c r="P183" s="8"/>
+      <x:c r="O183" s="9"/>
+      <x:c r="P183" s="9"/>
       <x:c r="Q183" s="8"/>
       <x:c r="R183" s="8"/>
       <x:c r="S183" s="8"/>
+      <x:c r="T183" s="8"/>
+      <x:c r="U183" s="8"/>
     </x:row>
     <x:row r="184" ht="20" customHeight="1">
       <x:c r="A184" s="8"/>
@@ -4223,11 +4619,13 @@
       <x:c r="L184" s="9"/>
       <x:c r="M184" s="9"/>
       <x:c r="N184" s="9"/>
-      <x:c r="O184" s="8"/>
-      <x:c r="P184" s="8"/>
+      <x:c r="O184" s="9"/>
+      <x:c r="P184" s="9"/>
       <x:c r="Q184" s="8"/>
       <x:c r="R184" s="8"/>
       <x:c r="S184" s="8"/>
+      <x:c r="T184" s="8"/>
+      <x:c r="U184" s="8"/>
     </x:row>
     <x:row r="185" ht="20" customHeight="1">
       <x:c r="A185" s="8"/>
@@ -4244,11 +4642,13 @@
       <x:c r="L185" s="9"/>
       <x:c r="M185" s="9"/>
       <x:c r="N185" s="9"/>
-      <x:c r="O185" s="8"/>
-      <x:c r="P185" s="8"/>
+      <x:c r="O185" s="9"/>
+      <x:c r="P185" s="9"/>
       <x:c r="Q185" s="8"/>
       <x:c r="R185" s="8"/>
       <x:c r="S185" s="8"/>
+      <x:c r="T185" s="8"/>
+      <x:c r="U185" s="8"/>
     </x:row>
     <x:row r="186" ht="20" customHeight="1">
       <x:c r="A186" s="8"/>
@@ -4265,11 +4665,13 @@
       <x:c r="L186" s="9"/>
       <x:c r="M186" s="9"/>
       <x:c r="N186" s="9"/>
-      <x:c r="O186" s="8"/>
-      <x:c r="P186" s="8"/>
+      <x:c r="O186" s="9"/>
+      <x:c r="P186" s="9"/>
       <x:c r="Q186" s="8"/>
       <x:c r="R186" s="8"/>
       <x:c r="S186" s="8"/>
+      <x:c r="T186" s="8"/>
+      <x:c r="U186" s="8"/>
     </x:row>
     <x:row r="187" ht="20" customHeight="1">
       <x:c r="A187" s="8"/>
@@ -4286,11 +4688,13 @@
       <x:c r="L187" s="9"/>
       <x:c r="M187" s="9"/>
       <x:c r="N187" s="9"/>
-      <x:c r="O187" s="8"/>
-      <x:c r="P187" s="8"/>
+      <x:c r="O187" s="9"/>
+      <x:c r="P187" s="9"/>
       <x:c r="Q187" s="8"/>
       <x:c r="R187" s="8"/>
       <x:c r="S187" s="8"/>
+      <x:c r="T187" s="8"/>
+      <x:c r="U187" s="8"/>
     </x:row>
     <x:row r="188" ht="20" customHeight="1">
       <x:c r="A188" s="8"/>
@@ -4307,11 +4711,13 @@
       <x:c r="L188" s="9"/>
       <x:c r="M188" s="9"/>
       <x:c r="N188" s="9"/>
-      <x:c r="O188" s="8"/>
-      <x:c r="P188" s="8"/>
+      <x:c r="O188" s="9"/>
+      <x:c r="P188" s="9"/>
       <x:c r="Q188" s="8"/>
       <x:c r="R188" s="8"/>
       <x:c r="S188" s="8"/>
+      <x:c r="T188" s="8"/>
+      <x:c r="U188" s="8"/>
     </x:row>
     <x:row r="189" ht="20" customHeight="1">
       <x:c r="A189" s="8"/>
@@ -4328,11 +4734,13 @@
       <x:c r="L189" s="9"/>
       <x:c r="M189" s="9"/>
       <x:c r="N189" s="9"/>
-      <x:c r="O189" s="8"/>
-      <x:c r="P189" s="8"/>
+      <x:c r="O189" s="9"/>
+      <x:c r="P189" s="9"/>
       <x:c r="Q189" s="8"/>
       <x:c r="R189" s="8"/>
       <x:c r="S189" s="8"/>
+      <x:c r="T189" s="8"/>
+      <x:c r="U189" s="8"/>
     </x:row>
     <x:row r="190" ht="20" customHeight="1">
       <x:c r="A190" s="8"/>
@@ -4349,11 +4757,13 @@
       <x:c r="L190" s="9"/>
       <x:c r="M190" s="9"/>
       <x:c r="N190" s="9"/>
-      <x:c r="O190" s="8"/>
-      <x:c r="P190" s="8"/>
+      <x:c r="O190" s="9"/>
+      <x:c r="P190" s="9"/>
       <x:c r="Q190" s="8"/>
       <x:c r="R190" s="8"/>
       <x:c r="S190" s="8"/>
+      <x:c r="T190" s="8"/>
+      <x:c r="U190" s="8"/>
     </x:row>
     <x:row r="191" ht="20" customHeight="1">
       <x:c r="A191" s="8"/>
@@ -4370,11 +4780,13 @@
       <x:c r="L191" s="9"/>
       <x:c r="M191" s="9"/>
       <x:c r="N191" s="9"/>
-      <x:c r="O191" s="8"/>
-      <x:c r="P191" s="8"/>
+      <x:c r="O191" s="9"/>
+      <x:c r="P191" s="9"/>
       <x:c r="Q191" s="8"/>
       <x:c r="R191" s="8"/>
       <x:c r="S191" s="8"/>
+      <x:c r="T191" s="8"/>
+      <x:c r="U191" s="8"/>
     </x:row>
     <x:row r="192" ht="20" customHeight="1">
       <x:c r="A192" s="8"/>
@@ -4391,11 +4803,13 @@
       <x:c r="L192" s="9"/>
       <x:c r="M192" s="9"/>
       <x:c r="N192" s="9"/>
-      <x:c r="O192" s="8"/>
-      <x:c r="P192" s="8"/>
+      <x:c r="O192" s="9"/>
+      <x:c r="P192" s="9"/>
       <x:c r="Q192" s="8"/>
       <x:c r="R192" s="8"/>
       <x:c r="S192" s="8"/>
+      <x:c r="T192" s="8"/>
+      <x:c r="U192" s="8"/>
     </x:row>
     <x:row r="193" ht="20" customHeight="1">
       <x:c r="A193" s="8"/>
@@ -4412,11 +4826,13 @@
       <x:c r="L193" s="9"/>
       <x:c r="M193" s="9"/>
       <x:c r="N193" s="9"/>
-      <x:c r="O193" s="8"/>
-      <x:c r="P193" s="8"/>
+      <x:c r="O193" s="9"/>
+      <x:c r="P193" s="9"/>
       <x:c r="Q193" s="8"/>
       <x:c r="R193" s="8"/>
       <x:c r="S193" s="8"/>
+      <x:c r="T193" s="8"/>
+      <x:c r="U193" s="8"/>
     </x:row>
     <x:row r="194" ht="20" customHeight="1">
       <x:c r="A194" s="8"/>
@@ -4433,11 +4849,13 @@
       <x:c r="L194" s="9"/>
       <x:c r="M194" s="9"/>
       <x:c r="N194" s="9"/>
-      <x:c r="O194" s="8"/>
-      <x:c r="P194" s="8"/>
+      <x:c r="O194" s="9"/>
+      <x:c r="P194" s="9"/>
       <x:c r="Q194" s="8"/>
       <x:c r="R194" s="8"/>
       <x:c r="S194" s="8"/>
+      <x:c r="T194" s="8"/>
+      <x:c r="U194" s="8"/>
     </x:row>
     <x:row r="195" ht="20" customHeight="1">
       <x:c r="A195" s="8"/>
@@ -4454,11 +4872,13 @@
       <x:c r="L195" s="9"/>
       <x:c r="M195" s="9"/>
       <x:c r="N195" s="9"/>
-      <x:c r="O195" s="8"/>
-      <x:c r="P195" s="8"/>
+      <x:c r="O195" s="9"/>
+      <x:c r="P195" s="9"/>
       <x:c r="Q195" s="8"/>
       <x:c r="R195" s="8"/>
       <x:c r="S195" s="8"/>
+      <x:c r="T195" s="8"/>
+      <x:c r="U195" s="8"/>
     </x:row>
     <x:row r="196" ht="20" customHeight="1">
       <x:c r="A196" s="8"/>
@@ -4475,11 +4895,13 @@
       <x:c r="L196" s="9"/>
       <x:c r="M196" s="9"/>
       <x:c r="N196" s="9"/>
-      <x:c r="O196" s="8"/>
-      <x:c r="P196" s="8"/>
+      <x:c r="O196" s="9"/>
+      <x:c r="P196" s="9"/>
       <x:c r="Q196" s="8"/>
       <x:c r="R196" s="8"/>
       <x:c r="S196" s="8"/>
+      <x:c r="T196" s="8"/>
+      <x:c r="U196" s="8"/>
     </x:row>
     <x:row r="197" ht="20" customHeight="1">
       <x:c r="A197" s="8"/>
@@ -4496,11 +4918,13 @@
       <x:c r="L197" s="9"/>
       <x:c r="M197" s="9"/>
       <x:c r="N197" s="9"/>
-      <x:c r="O197" s="8"/>
-      <x:c r="P197" s="8"/>
+      <x:c r="O197" s="9"/>
+      <x:c r="P197" s="9"/>
       <x:c r="Q197" s="8"/>
       <x:c r="R197" s="8"/>
       <x:c r="S197" s="8"/>
+      <x:c r="T197" s="8"/>
+      <x:c r="U197" s="8"/>
     </x:row>
     <x:row r="198" ht="20" customHeight="1">
       <x:c r="A198" s="8"/>
@@ -4517,11 +4941,13 @@
       <x:c r="L198" s="9"/>
       <x:c r="M198" s="9"/>
       <x:c r="N198" s="9"/>
-      <x:c r="O198" s="8"/>
-      <x:c r="P198" s="8"/>
+      <x:c r="O198" s="9"/>
+      <x:c r="P198" s="9"/>
       <x:c r="Q198" s="8"/>
       <x:c r="R198" s="8"/>
       <x:c r="S198" s="8"/>
+      <x:c r="T198" s="8"/>
+      <x:c r="U198" s="8"/>
     </x:row>
     <x:row r="199" ht="20" customHeight="1">
       <x:c r="A199" s="8"/>
@@ -4538,11 +4964,13 @@
       <x:c r="L199" s="9"/>
       <x:c r="M199" s="9"/>
       <x:c r="N199" s="9"/>
-      <x:c r="O199" s="8"/>
-      <x:c r="P199" s="8"/>
+      <x:c r="O199" s="9"/>
+      <x:c r="P199" s="9"/>
       <x:c r="Q199" s="8"/>
       <x:c r="R199" s="8"/>
       <x:c r="S199" s="8"/>
+      <x:c r="T199" s="8"/>
+      <x:c r="U199" s="8"/>
     </x:row>
     <x:row r="200" ht="20" customHeight="1">
       <x:c r="A200" s="8"/>
@@ -4559,11 +4987,13 @@
       <x:c r="L200" s="9"/>
       <x:c r="M200" s="9"/>
       <x:c r="N200" s="9"/>
-      <x:c r="O200" s="8"/>
-      <x:c r="P200" s="8"/>
+      <x:c r="O200" s="9"/>
+      <x:c r="P200" s="9"/>
       <x:c r="Q200" s="8"/>
       <x:c r="R200" s="8"/>
       <x:c r="S200" s="8"/>
+      <x:c r="T200" s="8"/>
+      <x:c r="U200" s="8"/>
     </x:row>
     <x:row r="201" ht="20" customHeight="1">
       <x:c r="A201" s="8"/>
@@ -4580,11 +5010,13 @@
       <x:c r="L201" s="9"/>
       <x:c r="M201" s="9"/>
       <x:c r="N201" s="9"/>
-      <x:c r="O201" s="8"/>
-      <x:c r="P201" s="8"/>
+      <x:c r="O201" s="9"/>
+      <x:c r="P201" s="9"/>
       <x:c r="Q201" s="8"/>
       <x:c r="R201" s="8"/>
       <x:c r="S201" s="8"/>
+      <x:c r="T201" s="8"/>
+      <x:c r="U201" s="8"/>
     </x:row>
     <x:row r="202" ht="20" customHeight="1">
       <x:c r="A202" s="8"/>
@@ -4601,11 +5033,13 @@
       <x:c r="L202" s="9"/>
       <x:c r="M202" s="9"/>
       <x:c r="N202" s="9"/>
-      <x:c r="O202" s="8"/>
-      <x:c r="P202" s="8"/>
+      <x:c r="O202" s="9"/>
+      <x:c r="P202" s="9"/>
       <x:c r="Q202" s="8"/>
       <x:c r="R202" s="8"/>
       <x:c r="S202" s="8"/>
+      <x:c r="T202" s="8"/>
+      <x:c r="U202" s="8"/>
     </x:row>
     <x:row r="203" ht="20" customHeight="1">
       <x:c r="A203" s="8"/>
@@ -4622,11 +5056,13 @@
       <x:c r="L203" s="9"/>
       <x:c r="M203" s="9"/>
       <x:c r="N203" s="9"/>
-      <x:c r="O203" s="8"/>
-      <x:c r="P203" s="8"/>
+      <x:c r="O203" s="9"/>
+      <x:c r="P203" s="9"/>
       <x:c r="Q203" s="8"/>
       <x:c r="R203" s="8"/>
       <x:c r="S203" s="8"/>
+      <x:c r="T203" s="8"/>
+      <x:c r="U203" s="8"/>
     </x:row>
     <x:row r="204" ht="20" customHeight="1">
       <x:c r="A204" s="8"/>
@@ -4643,11 +5079,13 @@
       <x:c r="L204" s="9"/>
       <x:c r="M204" s="9"/>
       <x:c r="N204" s="9"/>
-      <x:c r="O204" s="8"/>
-      <x:c r="P204" s="8"/>
+      <x:c r="O204" s="9"/>
+      <x:c r="P204" s="9"/>
       <x:c r="Q204" s="8"/>
       <x:c r="R204" s="8"/>
       <x:c r="S204" s="8"/>
+      <x:c r="T204" s="8"/>
+      <x:c r="U204" s="8"/>
     </x:row>
     <x:row r="205" ht="20" customHeight="1">
       <x:c r="A205" s="8"/>
@@ -4664,11 +5102,13 @@
       <x:c r="L205" s="9"/>
       <x:c r="M205" s="9"/>
       <x:c r="N205" s="9"/>
-      <x:c r="O205" s="8"/>
-      <x:c r="P205" s="8"/>
+      <x:c r="O205" s="9"/>
+      <x:c r="P205" s="9"/>
       <x:c r="Q205" s="8"/>
       <x:c r="R205" s="8"/>
       <x:c r="S205" s="8"/>
+      <x:c r="T205" s="8"/>
+      <x:c r="U205" s="8"/>
     </x:row>
     <x:row r="206" ht="20" customHeight="1">
       <x:c r="A206" s="8"/>
@@ -4685,11 +5125,13 @@
       <x:c r="L206" s="9"/>
       <x:c r="M206" s="9"/>
       <x:c r="N206" s="9"/>
-      <x:c r="O206" s="8"/>
-      <x:c r="P206" s="8"/>
+      <x:c r="O206" s="9"/>
+      <x:c r="P206" s="9"/>
       <x:c r="Q206" s="8"/>
       <x:c r="R206" s="8"/>
       <x:c r="S206" s="8"/>
+      <x:c r="T206" s="8"/>
+      <x:c r="U206" s="8"/>
     </x:row>
     <x:row r="207" ht="20" customHeight="1">
       <x:c r="A207" s="8"/>
@@ -4706,11 +5148,13 @@
       <x:c r="L207" s="9"/>
       <x:c r="M207" s="9"/>
       <x:c r="N207" s="9"/>
-      <x:c r="O207" s="8"/>
-      <x:c r="P207" s="8"/>
+      <x:c r="O207" s="9"/>
+      <x:c r="P207" s="9"/>
       <x:c r="Q207" s="8"/>
       <x:c r="R207" s="8"/>
       <x:c r="S207" s="8"/>
+      <x:c r="T207" s="8"/>
+      <x:c r="U207" s="8"/>
     </x:row>
     <x:row r="208" ht="20" customHeight="1">
       <x:c r="A208" s="8"/>
@@ -4727,11 +5171,13 @@
       <x:c r="L208" s="9"/>
       <x:c r="M208" s="9"/>
       <x:c r="N208" s="9"/>
-      <x:c r="O208" s="8"/>
-      <x:c r="P208" s="8"/>
+      <x:c r="O208" s="9"/>
+      <x:c r="P208" s="9"/>
       <x:c r="Q208" s="8"/>
       <x:c r="R208" s="8"/>
       <x:c r="S208" s="8"/>
+      <x:c r="T208" s="8"/>
+      <x:c r="U208" s="8"/>
     </x:row>
     <x:row r="209" ht="20" customHeight="1">
       <x:c r="A209" s="8"/>
@@ -4748,11 +5194,13 @@
       <x:c r="L209" s="9"/>
       <x:c r="M209" s="9"/>
       <x:c r="N209" s="9"/>
-      <x:c r="O209" s="8"/>
-      <x:c r="P209" s="8"/>
+      <x:c r="O209" s="9"/>
+      <x:c r="P209" s="9"/>
       <x:c r="Q209" s="8"/>
       <x:c r="R209" s="8"/>
       <x:c r="S209" s="8"/>
+      <x:c r="T209" s="8"/>
+      <x:c r="U209" s="8"/>
     </x:row>
     <x:row r="210" ht="20" customHeight="1">
       <x:c r="A210" s="8"/>
@@ -4769,11 +5217,13 @@
       <x:c r="L210" s="9"/>
       <x:c r="M210" s="9"/>
       <x:c r="N210" s="9"/>
-      <x:c r="O210" s="8"/>
-      <x:c r="P210" s="8"/>
+      <x:c r="O210" s="9"/>
+      <x:c r="P210" s="9"/>
       <x:c r="Q210" s="8"/>
       <x:c r="R210" s="8"/>
       <x:c r="S210" s="8"/>
+      <x:c r="T210" s="8"/>
+      <x:c r="U210" s="8"/>
     </x:row>
     <x:row r="211" ht="20" customHeight="1">
       <x:c r="A211" s="8"/>
@@ -4790,11 +5240,13 @@
       <x:c r="L211" s="9"/>
       <x:c r="M211" s="9"/>
       <x:c r="N211" s="9"/>
-      <x:c r="O211" s="8"/>
-      <x:c r="P211" s="8"/>
+      <x:c r="O211" s="9"/>
+      <x:c r="P211" s="9"/>
       <x:c r="Q211" s="8"/>
       <x:c r="R211" s="8"/>
       <x:c r="S211" s="8"/>
+      <x:c r="T211" s="8"/>
+      <x:c r="U211" s="8"/>
     </x:row>
     <x:row r="212" ht="20" customHeight="1">
       <x:c r="A212" s="8"/>
@@ -4811,11 +5263,13 @@
       <x:c r="L212" s="9"/>
       <x:c r="M212" s="9"/>
       <x:c r="N212" s="9"/>
-      <x:c r="O212" s="8"/>
-      <x:c r="P212" s="8"/>
+      <x:c r="O212" s="9"/>
+      <x:c r="P212" s="9"/>
       <x:c r="Q212" s="8"/>
       <x:c r="R212" s="8"/>
       <x:c r="S212" s="8"/>
+      <x:c r="T212" s="8"/>
+      <x:c r="U212" s="8"/>
     </x:row>
     <x:row r="213" ht="20" customHeight="1">
       <x:c r="A213" s="8"/>
@@ -4832,11 +5286,13 @@
       <x:c r="L213" s="9"/>
       <x:c r="M213" s="9"/>
       <x:c r="N213" s="9"/>
-      <x:c r="O213" s="8"/>
-      <x:c r="P213" s="8"/>
+      <x:c r="O213" s="9"/>
+      <x:c r="P213" s="9"/>
       <x:c r="Q213" s="8"/>
       <x:c r="R213" s="8"/>
       <x:c r="S213" s="8"/>
+      <x:c r="T213" s="8"/>
+      <x:c r="U213" s="8"/>
     </x:row>
     <x:row r="214" ht="20" customHeight="1">
       <x:c r="A214" s="8"/>
@@ -4853,11 +5309,13 @@
       <x:c r="L214" s="9"/>
       <x:c r="M214" s="9"/>
       <x:c r="N214" s="9"/>
-      <x:c r="O214" s="8"/>
-      <x:c r="P214" s="8"/>
+      <x:c r="O214" s="9"/>
+      <x:c r="P214" s="9"/>
       <x:c r="Q214" s="8"/>
       <x:c r="R214" s="8"/>
       <x:c r="S214" s="8"/>
+      <x:c r="T214" s="8"/>
+      <x:c r="U214" s="8"/>
     </x:row>
     <x:row r="215" ht="20" customHeight="1">
       <x:c r="A215" s="8"/>
@@ -4874,11 +5332,13 @@
       <x:c r="L215" s="9"/>
       <x:c r="M215" s="9"/>
       <x:c r="N215" s="9"/>
-      <x:c r="O215" s="8"/>
-      <x:c r="P215" s="8"/>
+      <x:c r="O215" s="9"/>
+      <x:c r="P215" s="9"/>
       <x:c r="Q215" s="8"/>
       <x:c r="R215" s="8"/>
       <x:c r="S215" s="8"/>
+      <x:c r="T215" s="8"/>
+      <x:c r="U215" s="8"/>
     </x:row>
     <x:row r="216" ht="20" customHeight="1">
       <x:c r="A216" s="8"/>
@@ -4895,11 +5355,13 @@
       <x:c r="L216" s="9"/>
       <x:c r="M216" s="9"/>
       <x:c r="N216" s="9"/>
-      <x:c r="O216" s="8"/>
-      <x:c r="P216" s="8"/>
+      <x:c r="O216" s="9"/>
+      <x:c r="P216" s="9"/>
       <x:c r="Q216" s="8"/>
       <x:c r="R216" s="8"/>
       <x:c r="S216" s="8"/>
+      <x:c r="T216" s="8"/>
+      <x:c r="U216" s="8"/>
     </x:row>
     <x:row r="217" ht="20" customHeight="1">
       <x:c r="A217" s="8"/>
@@ -4916,11 +5378,13 @@
       <x:c r="L217" s="9"/>
       <x:c r="M217" s="9"/>
       <x:c r="N217" s="9"/>
-      <x:c r="O217" s="8"/>
-      <x:c r="P217" s="8"/>
+      <x:c r="O217" s="9"/>
+      <x:c r="P217" s="9"/>
       <x:c r="Q217" s="8"/>
       <x:c r="R217" s="8"/>
       <x:c r="S217" s="8"/>
+      <x:c r="T217" s="8"/>
+      <x:c r="U217" s="8"/>
     </x:row>
     <x:row r="218" ht="20" customHeight="1">
       <x:c r="A218" s="8"/>
@@ -4937,11 +5401,13 @@
       <x:c r="L218" s="9"/>
       <x:c r="M218" s="9"/>
       <x:c r="N218" s="9"/>
-      <x:c r="O218" s="8"/>
-      <x:c r="P218" s="8"/>
+      <x:c r="O218" s="9"/>
+      <x:c r="P218" s="9"/>
       <x:c r="Q218" s="8"/>
       <x:c r="R218" s="8"/>
       <x:c r="S218" s="8"/>
+      <x:c r="T218" s="8"/>
+      <x:c r="U218" s="8"/>
     </x:row>
     <x:row r="219" ht="20" customHeight="1">
       <x:c r="A219" s="8"/>
@@ -4958,11 +5424,13 @@
       <x:c r="L219" s="9"/>
       <x:c r="M219" s="9"/>
       <x:c r="N219" s="9"/>
-      <x:c r="O219" s="8"/>
-      <x:c r="P219" s="8"/>
+      <x:c r="O219" s="9"/>
+      <x:c r="P219" s="9"/>
       <x:c r="Q219" s="8"/>
       <x:c r="R219" s="8"/>
       <x:c r="S219" s="8"/>
+      <x:c r="T219" s="8"/>
+      <x:c r="U219" s="8"/>
     </x:row>
     <x:row r="220" ht="20" customHeight="1">
       <x:c r="A220" s="8"/>
@@ -4979,11 +5447,13 @@
       <x:c r="L220" s="9"/>
       <x:c r="M220" s="9"/>
       <x:c r="N220" s="9"/>
-      <x:c r="O220" s="8"/>
-      <x:c r="P220" s="8"/>
+      <x:c r="O220" s="9"/>
+      <x:c r="P220" s="9"/>
       <x:c r="Q220" s="8"/>
       <x:c r="R220" s="8"/>
       <x:c r="S220" s="8"/>
+      <x:c r="T220" s="8"/>
+      <x:c r="U220" s="8"/>
     </x:row>
     <x:row r="221" ht="20" customHeight="1">
       <x:c r="A221" s="8"/>
@@ -5000,11 +5470,13 @@
       <x:c r="L221" s="9"/>
       <x:c r="M221" s="9"/>
       <x:c r="N221" s="9"/>
-      <x:c r="O221" s="8"/>
-      <x:c r="P221" s="8"/>
+      <x:c r="O221" s="9"/>
+      <x:c r="P221" s="9"/>
       <x:c r="Q221" s="8"/>
       <x:c r="R221" s="8"/>
       <x:c r="S221" s="8"/>
+      <x:c r="T221" s="8"/>
+      <x:c r="U221" s="8"/>
     </x:row>
     <x:row r="222" ht="20" customHeight="1">
       <x:c r="A222" s="8"/>
@@ -5021,11 +5493,13 @@
       <x:c r="L222" s="9"/>
       <x:c r="M222" s="9"/>
       <x:c r="N222" s="9"/>
-      <x:c r="O222" s="8"/>
-      <x:c r="P222" s="8"/>
+      <x:c r="O222" s="9"/>
+      <x:c r="P222" s="9"/>
       <x:c r="Q222" s="8"/>
       <x:c r="R222" s="8"/>
       <x:c r="S222" s="8"/>
+      <x:c r="T222" s="8"/>
+      <x:c r="U222" s="8"/>
     </x:row>
     <x:row r="223" ht="20" customHeight="1">
       <x:c r="A223" s="8"/>
@@ -5042,11 +5516,13 @@
       <x:c r="L223" s="9"/>
       <x:c r="M223" s="9"/>
       <x:c r="N223" s="9"/>
-      <x:c r="O223" s="8"/>
-      <x:c r="P223" s="8"/>
+      <x:c r="O223" s="9"/>
+      <x:c r="P223" s="9"/>
       <x:c r="Q223" s="8"/>
       <x:c r="R223" s="8"/>
       <x:c r="S223" s="8"/>
+      <x:c r="T223" s="8"/>
+      <x:c r="U223" s="8"/>
     </x:row>
     <x:row r="224" ht="20" customHeight="1">
       <x:c r="A224" s="8"/>
@@ -5063,11 +5539,13 @@
       <x:c r="L224" s="9"/>
       <x:c r="M224" s="9"/>
       <x:c r="N224" s="9"/>
-      <x:c r="O224" s="8"/>
-      <x:c r="P224" s="8"/>
+      <x:c r="O224" s="9"/>
+      <x:c r="P224" s="9"/>
       <x:c r="Q224" s="8"/>
       <x:c r="R224" s="8"/>
       <x:c r="S224" s="8"/>
+      <x:c r="T224" s="8"/>
+      <x:c r="U224" s="8"/>
     </x:row>
     <x:row r="225" ht="20" customHeight="1">
       <x:c r="A225" s="8"/>
@@ -5084,11 +5562,13 @@
       <x:c r="L225" s="9"/>
       <x:c r="M225" s="9"/>
       <x:c r="N225" s="9"/>
-      <x:c r="O225" s="8"/>
-      <x:c r="P225" s="8"/>
+      <x:c r="O225" s="9"/>
+      <x:c r="P225" s="9"/>
       <x:c r="Q225" s="8"/>
       <x:c r="R225" s="8"/>
       <x:c r="S225" s="8"/>
+      <x:c r="T225" s="8"/>
+      <x:c r="U225" s="8"/>
     </x:row>
     <x:row r="226" ht="20" customHeight="1">
       <x:c r="A226" s="8"/>
@@ -5105,11 +5585,13 @@
       <x:c r="L226" s="9"/>
       <x:c r="M226" s="9"/>
       <x:c r="N226" s="9"/>
-      <x:c r="O226" s="8"/>
-      <x:c r="P226" s="8"/>
+      <x:c r="O226" s="9"/>
+      <x:c r="P226" s="9"/>
       <x:c r="Q226" s="8"/>
       <x:c r="R226" s="8"/>
       <x:c r="S226" s="8"/>
+      <x:c r="T226" s="8"/>
+      <x:c r="U226" s="8"/>
     </x:row>
     <x:row r="227" ht="20" customHeight="1">
       <x:c r="A227" s="8"/>
@@ -5126,11 +5608,13 @@
       <x:c r="L227" s="9"/>
       <x:c r="M227" s="9"/>
       <x:c r="N227" s="9"/>
-      <x:c r="O227" s="8"/>
-      <x:c r="P227" s="8"/>
+      <x:c r="O227" s="9"/>
+      <x:c r="P227" s="9"/>
       <x:c r="Q227" s="8"/>
       <x:c r="R227" s="8"/>
       <x:c r="S227" s="8"/>
+      <x:c r="T227" s="8"/>
+      <x:c r="U227" s="8"/>
     </x:row>
     <x:row r="228" ht="20" customHeight="1">
       <x:c r="A228" s="8"/>
@@ -5147,11 +5631,13 @@
       <x:c r="L228" s="9"/>
       <x:c r="M228" s="9"/>
       <x:c r="N228" s="9"/>
-      <x:c r="O228" s="8"/>
-      <x:c r="P228" s="8"/>
+      <x:c r="O228" s="9"/>
+      <x:c r="P228" s="9"/>
       <x:c r="Q228" s="8"/>
       <x:c r="R228" s="8"/>
       <x:c r="S228" s="8"/>
+      <x:c r="T228" s="8"/>
+      <x:c r="U228" s="8"/>
     </x:row>
     <x:row r="229" ht="20" customHeight="1">
       <x:c r="A229" s="8"/>
@@ -5168,11 +5654,13 @@
       <x:c r="L229" s="9"/>
       <x:c r="M229" s="9"/>
       <x:c r="N229" s="9"/>
-      <x:c r="O229" s="8"/>
-      <x:c r="P229" s="8"/>
+      <x:c r="O229" s="9"/>
+      <x:c r="P229" s="9"/>
       <x:c r="Q229" s="8"/>
       <x:c r="R229" s="8"/>
       <x:c r="S229" s="8"/>
+      <x:c r="T229" s="8"/>
+      <x:c r="U229" s="8"/>
     </x:row>
     <x:row r="230" ht="20" customHeight="1">
       <x:c r="A230" s="8"/>
@@ -5189,11 +5677,13 @@
       <x:c r="L230" s="9"/>
       <x:c r="M230" s="9"/>
       <x:c r="N230" s="9"/>
-      <x:c r="O230" s="8"/>
-      <x:c r="P230" s="8"/>
+      <x:c r="O230" s="9"/>
+      <x:c r="P230" s="9"/>
       <x:c r="Q230" s="8"/>
       <x:c r="R230" s="8"/>
       <x:c r="S230" s="8"/>
+      <x:c r="T230" s="8"/>
+      <x:c r="U230" s="8"/>
     </x:row>
     <x:row r="231" ht="20" customHeight="1">
       <x:c r="A231" s="8"/>
@@ -5210,11 +5700,13 @@
       <x:c r="L231" s="9"/>
       <x:c r="M231" s="9"/>
       <x:c r="N231" s="9"/>
-      <x:c r="O231" s="8"/>
-      <x:c r="P231" s="8"/>
+      <x:c r="O231" s="9"/>
+      <x:c r="P231" s="9"/>
       <x:c r="Q231" s="8"/>
       <x:c r="R231" s="8"/>
       <x:c r="S231" s="8"/>
+      <x:c r="T231" s="8"/>
+      <x:c r="U231" s="8"/>
     </x:row>
     <x:row r="232" ht="20" customHeight="1">
       <x:c r="A232" s="8"/>
@@ -5231,11 +5723,13 @@
       <x:c r="L232" s="9"/>
       <x:c r="M232" s="9"/>
       <x:c r="N232" s="9"/>
-      <x:c r="O232" s="8"/>
-      <x:c r="P232" s="8"/>
+      <x:c r="O232" s="9"/>
+      <x:c r="P232" s="9"/>
       <x:c r="Q232" s="8"/>
       <x:c r="R232" s="8"/>
       <x:c r="S232" s="8"/>
+      <x:c r="T232" s="8"/>
+      <x:c r="U232" s="8"/>
     </x:row>
     <x:row r="233" ht="20" customHeight="1">
       <x:c r="A233" s="8"/>
@@ -5252,11 +5746,13 @@
       <x:c r="L233" s="9"/>
       <x:c r="M233" s="9"/>
       <x:c r="N233" s="9"/>
-      <x:c r="O233" s="8"/>
-      <x:c r="P233" s="8"/>
+      <x:c r="O233" s="9"/>
+      <x:c r="P233" s="9"/>
       <x:c r="Q233" s="8"/>
       <x:c r="R233" s="8"/>
       <x:c r="S233" s="8"/>
+      <x:c r="T233" s="8"/>
+      <x:c r="U233" s="8"/>
     </x:row>
     <x:row r="234" ht="20" customHeight="1">
       <x:c r="A234" s="8"/>
@@ -5273,11 +5769,13 @@
       <x:c r="L234" s="9"/>
       <x:c r="M234" s="9"/>
       <x:c r="N234" s="9"/>
-      <x:c r="O234" s="8"/>
-      <x:c r="P234" s="8"/>
+      <x:c r="O234" s="9"/>
+      <x:c r="P234" s="9"/>
       <x:c r="Q234" s="8"/>
       <x:c r="R234" s="8"/>
       <x:c r="S234" s="8"/>
+      <x:c r="T234" s="8"/>
+      <x:c r="U234" s="8"/>
     </x:row>
     <x:row r="235" ht="20" customHeight="1">
       <x:c r="A235" s="8"/>
@@ -5294,11 +5792,13 @@
       <x:c r="L235" s="9"/>
       <x:c r="M235" s="9"/>
       <x:c r="N235" s="9"/>
-      <x:c r="O235" s="8"/>
-      <x:c r="P235" s="8"/>
+      <x:c r="O235" s="9"/>
+      <x:c r="P235" s="9"/>
       <x:c r="Q235" s="8"/>
       <x:c r="R235" s="8"/>
       <x:c r="S235" s="8"/>
+      <x:c r="T235" s="8"/>
+      <x:c r="U235" s="8"/>
     </x:row>
     <x:row r="236" ht="20" customHeight="1">
       <x:c r="A236" s="8"/>
@@ -5315,11 +5815,13 @@
       <x:c r="L236" s="9"/>
       <x:c r="M236" s="9"/>
       <x:c r="N236" s="9"/>
-      <x:c r="O236" s="8"/>
-      <x:c r="P236" s="8"/>
+      <x:c r="O236" s="9"/>
+      <x:c r="P236" s="9"/>
       <x:c r="Q236" s="8"/>
       <x:c r="R236" s="8"/>
       <x:c r="S236" s="8"/>
+      <x:c r="T236" s="8"/>
+      <x:c r="U236" s="8"/>
     </x:row>
     <x:row r="237" ht="20" customHeight="1">
       <x:c r="A237" s="8"/>
@@ -5336,11 +5838,13 @@
       <x:c r="L237" s="9"/>
       <x:c r="M237" s="9"/>
       <x:c r="N237" s="9"/>
-      <x:c r="O237" s="8"/>
-      <x:c r="P237" s="8"/>
+      <x:c r="O237" s="9"/>
+      <x:c r="P237" s="9"/>
       <x:c r="Q237" s="8"/>
       <x:c r="R237" s="8"/>
       <x:c r="S237" s="8"/>
+      <x:c r="T237" s="8"/>
+      <x:c r="U237" s="8"/>
     </x:row>
     <x:row r="238" ht="20" customHeight="1">
       <x:c r="A238" s="8"/>
@@ -5357,11 +5861,13 @@
       <x:c r="L238" s="9"/>
       <x:c r="M238" s="9"/>
       <x:c r="N238" s="9"/>
-      <x:c r="O238" s="8"/>
-      <x:c r="P238" s="8"/>
+      <x:c r="O238" s="9"/>
+      <x:c r="P238" s="9"/>
       <x:c r="Q238" s="8"/>
       <x:c r="R238" s="8"/>
       <x:c r="S238" s="8"/>
+      <x:c r="T238" s="8"/>
+      <x:c r="U238" s="8"/>
     </x:row>
     <x:row r="239" ht="20" customHeight="1">
       <x:c r="A239" s="8"/>
@@ -5378,11 +5884,13 @@
       <x:c r="L239" s="9"/>
       <x:c r="M239" s="9"/>
       <x:c r="N239" s="9"/>
-      <x:c r="O239" s="8"/>
-      <x:c r="P239" s="8"/>
+      <x:c r="O239" s="9"/>
+      <x:c r="P239" s="9"/>
       <x:c r="Q239" s="8"/>
       <x:c r="R239" s="8"/>
       <x:c r="S239" s="8"/>
+      <x:c r="T239" s="8"/>
+      <x:c r="U239" s="8"/>
     </x:row>
     <x:row r="240" ht="20" customHeight="1">
       <x:c r="A240" s="8"/>
@@ -5399,11 +5907,13 @@
       <x:c r="L240" s="9"/>
       <x:c r="M240" s="9"/>
       <x:c r="N240" s="9"/>
-      <x:c r="O240" s="8"/>
-      <x:c r="P240" s="8"/>
+      <x:c r="O240" s="9"/>
+      <x:c r="P240" s="9"/>
       <x:c r="Q240" s="8"/>
       <x:c r="R240" s="8"/>
       <x:c r="S240" s="8"/>
+      <x:c r="T240" s="8"/>
+      <x:c r="U240" s="8"/>
     </x:row>
     <x:row r="241" ht="20" customHeight="1">
       <x:c r="A241" s="8"/>
@@ -5420,11 +5930,13 @@
       <x:c r="L241" s="9"/>
       <x:c r="M241" s="9"/>
       <x:c r="N241" s="9"/>
-      <x:c r="O241" s="8"/>
-      <x:c r="P241" s="8"/>
+      <x:c r="O241" s="9"/>
+      <x:c r="P241" s="9"/>
       <x:c r="Q241" s="8"/>
       <x:c r="R241" s="8"/>
       <x:c r="S241" s="8"/>
+      <x:c r="T241" s="8"/>
+      <x:c r="U241" s="8"/>
     </x:row>
     <x:row r="242" ht="20" customHeight="1">
       <x:c r="A242" s="8"/>
@@ -5441,11 +5953,13 @@
       <x:c r="L242" s="9"/>
       <x:c r="M242" s="9"/>
       <x:c r="N242" s="9"/>
-      <x:c r="O242" s="8"/>
-      <x:c r="P242" s="8"/>
+      <x:c r="O242" s="9"/>
+      <x:c r="P242" s="9"/>
       <x:c r="Q242" s="8"/>
       <x:c r="R242" s="8"/>
       <x:c r="S242" s="8"/>
+      <x:c r="T242" s="8"/>
+      <x:c r="U242" s="8"/>
     </x:row>
     <x:row r="243" ht="20" customHeight="1">
       <x:c r="A243" s="8"/>
@@ -5462,11 +5976,13 @@
       <x:c r="L243" s="9"/>
       <x:c r="M243" s="9"/>
       <x:c r="N243" s="9"/>
-      <x:c r="O243" s="8"/>
-      <x:c r="P243" s="8"/>
+      <x:c r="O243" s="9"/>
+      <x:c r="P243" s="9"/>
       <x:c r="Q243" s="8"/>
       <x:c r="R243" s="8"/>
       <x:c r="S243" s="8"/>
+      <x:c r="T243" s="8"/>
+      <x:c r="U243" s="8"/>
     </x:row>
     <x:row r="244" ht="20" customHeight="1">
       <x:c r="A244" s="8"/>
@@ -5483,11 +5999,13 @@
       <x:c r="L244" s="9"/>
       <x:c r="M244" s="9"/>
       <x:c r="N244" s="9"/>
-      <x:c r="O244" s="8"/>
-      <x:c r="P244" s="8"/>
+      <x:c r="O244" s="9"/>
+      <x:c r="P244" s="9"/>
       <x:c r="Q244" s="8"/>
       <x:c r="R244" s="8"/>
       <x:c r="S244" s="8"/>
+      <x:c r="T244" s="8"/>
+      <x:c r="U244" s="8"/>
     </x:row>
     <x:row r="245" ht="20" customHeight="1">
       <x:c r="A245" s="8"/>
@@ -5504,11 +6022,13 @@
       <x:c r="L245" s="9"/>
       <x:c r="M245" s="9"/>
       <x:c r="N245" s="9"/>
-      <x:c r="O245" s="8"/>
-      <x:c r="P245" s="8"/>
+      <x:c r="O245" s="9"/>
+      <x:c r="P245" s="9"/>
       <x:c r="Q245" s="8"/>
       <x:c r="R245" s="8"/>
       <x:c r="S245" s="8"/>
+      <x:c r="T245" s="8"/>
+      <x:c r="U245" s="8"/>
     </x:row>
     <x:row r="246" ht="20" customHeight="1">
       <x:c r="A246" s="8"/>
@@ -5525,11 +6045,13 @@
       <x:c r="L246" s="9"/>
       <x:c r="M246" s="9"/>
       <x:c r="N246" s="9"/>
-      <x:c r="O246" s="8"/>
-      <x:c r="P246" s="8"/>
+      <x:c r="O246" s="9"/>
+      <x:c r="P246" s="9"/>
       <x:c r="Q246" s="8"/>
       <x:c r="R246" s="8"/>
       <x:c r="S246" s="8"/>
+      <x:c r="T246" s="8"/>
+      <x:c r="U246" s="8"/>
     </x:row>
     <x:row r="247" ht="20" customHeight="1">
       <x:c r="A247" s="8"/>
@@ -5546,11 +6068,13 @@
       <x:c r="L247" s="9"/>
       <x:c r="M247" s="9"/>
       <x:c r="N247" s="9"/>
-      <x:c r="O247" s="8"/>
-      <x:c r="P247" s="8"/>
+      <x:c r="O247" s="9"/>
+      <x:c r="P247" s="9"/>
       <x:c r="Q247" s="8"/>
       <x:c r="R247" s="8"/>
       <x:c r="S247" s="8"/>
+      <x:c r="T247" s="8"/>
+      <x:c r="U247" s="8"/>
     </x:row>
     <x:row r="248" ht="20" customHeight="1">
       <x:c r="A248" s="8"/>
@@ -5567,11 +6091,13 @@
       <x:c r="L248" s="9"/>
       <x:c r="M248" s="9"/>
       <x:c r="N248" s="9"/>
-      <x:c r="O248" s="8"/>
-      <x:c r="P248" s="8"/>
+      <x:c r="O248" s="9"/>
+      <x:c r="P248" s="9"/>
       <x:c r="Q248" s="8"/>
       <x:c r="R248" s="8"/>
       <x:c r="S248" s="8"/>
+      <x:c r="T248" s="8"/>
+      <x:c r="U248" s="8"/>
     </x:row>
     <x:row r="249" ht="20" customHeight="1">
       <x:c r="A249" s="8"/>
@@ -5588,11 +6114,13 @@
       <x:c r="L249" s="9"/>
       <x:c r="M249" s="9"/>
       <x:c r="N249" s="9"/>
-      <x:c r="O249" s="8"/>
-      <x:c r="P249" s="8"/>
+      <x:c r="O249" s="9"/>
+      <x:c r="P249" s="9"/>
       <x:c r="Q249" s="8"/>
       <x:c r="R249" s="8"/>
       <x:c r="S249" s="8"/>
+      <x:c r="T249" s="8"/>
+      <x:c r="U249" s="8"/>
     </x:row>
     <x:row r="250" ht="20" customHeight="1">
       <x:c r="A250" s="8"/>
@@ -5609,11 +6137,13 @@
       <x:c r="L250" s="9"/>
       <x:c r="M250" s="9"/>
       <x:c r="N250" s="9"/>
-      <x:c r="O250" s="8"/>
-      <x:c r="P250" s="8"/>
+      <x:c r="O250" s="9"/>
+      <x:c r="P250" s="9"/>
       <x:c r="Q250" s="8"/>
       <x:c r="R250" s="8"/>
       <x:c r="S250" s="8"/>
+      <x:c r="T250" s="8"/>
+      <x:c r="U250" s="8"/>
     </x:row>
     <x:row r="251" ht="20" customHeight="1">
       <x:c r="A251" s="8"/>
@@ -5630,11 +6160,13 @@
       <x:c r="L251" s="9"/>
       <x:c r="M251" s="9"/>
       <x:c r="N251" s="9"/>
-      <x:c r="O251" s="8"/>
-      <x:c r="P251" s="8"/>
+      <x:c r="O251" s="9"/>
+      <x:c r="P251" s="9"/>
       <x:c r="Q251" s="8"/>
       <x:c r="R251" s="8"/>
       <x:c r="S251" s="8"/>
+      <x:c r="T251" s="8"/>
+      <x:c r="U251" s="8"/>
     </x:row>
     <x:row r="252" ht="20" customHeight="1">
       <x:c r="A252" s="8"/>
@@ -5651,11 +6183,13 @@
       <x:c r="L252" s="9"/>
       <x:c r="M252" s="9"/>
       <x:c r="N252" s="9"/>
-      <x:c r="O252" s="8"/>
-      <x:c r="P252" s="8"/>
+      <x:c r="O252" s="9"/>
+      <x:c r="P252" s="9"/>
       <x:c r="Q252" s="8"/>
       <x:c r="R252" s="8"/>
       <x:c r="S252" s="8"/>
+      <x:c r="T252" s="8"/>
+      <x:c r="U252" s="8"/>
     </x:row>
     <x:row r="253" ht="20" customHeight="1">
       <x:c r="A253" s="8"/>
@@ -5672,11 +6206,13 @@
       <x:c r="L253" s="9"/>
       <x:c r="M253" s="9"/>
       <x:c r="N253" s="9"/>
-      <x:c r="O253" s="8"/>
-      <x:c r="P253" s="8"/>
+      <x:c r="O253" s="9"/>
+      <x:c r="P253" s="9"/>
       <x:c r="Q253" s="8"/>
       <x:c r="R253" s="8"/>
       <x:c r="S253" s="8"/>
+      <x:c r="T253" s="8"/>
+      <x:c r="U253" s="8"/>
     </x:row>
     <x:row r="254" ht="20" customHeight="1">
       <x:c r="A254" s="8"/>
@@ -5693,11 +6229,13 @@
       <x:c r="L254" s="9"/>
       <x:c r="M254" s="9"/>
       <x:c r="N254" s="9"/>
-      <x:c r="O254" s="8"/>
-      <x:c r="P254" s="8"/>
+      <x:c r="O254" s="9"/>
+      <x:c r="P254" s="9"/>
       <x:c r="Q254" s="8"/>
       <x:c r="R254" s="8"/>
       <x:c r="S254" s="8"/>
+      <x:c r="T254" s="8"/>
+      <x:c r="U254" s="8"/>
     </x:row>
     <x:row r="255" ht="20" customHeight="1">
       <x:c r="A255" s="8"/>
@@ -5714,11 +6252,13 @@
       <x:c r="L255" s="9"/>
       <x:c r="M255" s="9"/>
       <x:c r="N255" s="9"/>
-      <x:c r="O255" s="8"/>
-      <x:c r="P255" s="8"/>
+      <x:c r="O255" s="9"/>
+      <x:c r="P255" s="9"/>
       <x:c r="Q255" s="8"/>
       <x:c r="R255" s="8"/>
       <x:c r="S255" s="8"/>
+      <x:c r="T255" s="8"/>
+      <x:c r="U255" s="8"/>
     </x:row>
     <x:row r="256" ht="20" customHeight="1">
       <x:c r="A256" s="8"/>
@@ -5735,11 +6275,13 @@
       <x:c r="L256" s="9"/>
       <x:c r="M256" s="9"/>
       <x:c r="N256" s="9"/>
-      <x:c r="O256" s="8"/>
-      <x:c r="P256" s="8"/>
+      <x:c r="O256" s="9"/>
+      <x:c r="P256" s="9"/>
       <x:c r="Q256" s="8"/>
       <x:c r="R256" s="8"/>
       <x:c r="S256" s="8"/>
+      <x:c r="T256" s="8"/>
+      <x:c r="U256" s="8"/>
     </x:row>
     <x:row r="257" ht="20" customHeight="1">
       <x:c r="A257" s="8"/>
@@ -5756,11 +6298,13 @@
       <x:c r="L257" s="9"/>
       <x:c r="M257" s="9"/>
       <x:c r="N257" s="9"/>
-      <x:c r="O257" s="8"/>
-      <x:c r="P257" s="8"/>
+      <x:c r="O257" s="9"/>
+      <x:c r="P257" s="9"/>
       <x:c r="Q257" s="8"/>
       <x:c r="R257" s="8"/>
       <x:c r="S257" s="8"/>
+      <x:c r="T257" s="8"/>
+      <x:c r="U257" s="8"/>
     </x:row>
     <x:row r="258" ht="20" customHeight="1">
       <x:c r="A258" s="8"/>
@@ -5777,11 +6321,13 @@
       <x:c r="L258" s="9"/>
       <x:c r="M258" s="9"/>
       <x:c r="N258" s="9"/>
-      <x:c r="O258" s="8"/>
-      <x:c r="P258" s="8"/>
+      <x:c r="O258" s="9"/>
+      <x:c r="P258" s="9"/>
       <x:c r="Q258" s="8"/>
       <x:c r="R258" s="8"/>
       <x:c r="S258" s="8"/>
+      <x:c r="T258" s="8"/>
+      <x:c r="U258" s="8"/>
     </x:row>
     <x:row r="259" ht="20" customHeight="1">
       <x:c r="A259" s="8"/>
@@ -5798,11 +6344,13 @@
       <x:c r="L259" s="9"/>
       <x:c r="M259" s="9"/>
       <x:c r="N259" s="9"/>
-      <x:c r="O259" s="8"/>
-      <x:c r="P259" s="8"/>
+      <x:c r="O259" s="9"/>
+      <x:c r="P259" s="9"/>
       <x:c r="Q259" s="8"/>
       <x:c r="R259" s="8"/>
       <x:c r="S259" s="8"/>
+      <x:c r="T259" s="8"/>
+      <x:c r="U259" s="8"/>
     </x:row>
     <x:row r="260" ht="20" customHeight="1">
       <x:c r="A260" s="8"/>
@@ -5819,11 +6367,13 @@
       <x:c r="L260" s="9"/>
       <x:c r="M260" s="9"/>
       <x:c r="N260" s="9"/>
-      <x:c r="O260" s="8"/>
-      <x:c r="P260" s="8"/>
+      <x:c r="O260" s="9"/>
+      <x:c r="P260" s="9"/>
       <x:c r="Q260" s="8"/>
       <x:c r="R260" s="8"/>
       <x:c r="S260" s="8"/>
+      <x:c r="T260" s="8"/>
+      <x:c r="U260" s="8"/>
     </x:row>
     <x:row r="261" ht="20" customHeight="1">
       <x:c r="A261" s="8"/>
@@ -5840,11 +6390,13 @@
       <x:c r="L261" s="9"/>
       <x:c r="M261" s="9"/>
       <x:c r="N261" s="9"/>
-      <x:c r="O261" s="8"/>
-      <x:c r="P261" s="8"/>
+      <x:c r="O261" s="9"/>
+      <x:c r="P261" s="9"/>
       <x:c r="Q261" s="8"/>
       <x:c r="R261" s="8"/>
       <x:c r="S261" s="8"/>
+      <x:c r="T261" s="8"/>
+      <x:c r="U261" s="8"/>
     </x:row>
     <x:row r="262" ht="20" customHeight="1">
       <x:c r="A262" s="8"/>
@@ -5861,11 +6413,13 @@
       <x:c r="L262" s="9"/>
       <x:c r="M262" s="9"/>
       <x:c r="N262" s="9"/>
-      <x:c r="O262" s="8"/>
-      <x:c r="P262" s="8"/>
+      <x:c r="O262" s="9"/>
+      <x:c r="P262" s="9"/>
       <x:c r="Q262" s="8"/>
       <x:c r="R262" s="8"/>
       <x:c r="S262" s="8"/>
+      <x:c r="T262" s="8"/>
+      <x:c r="U262" s="8"/>
     </x:row>
     <x:row r="263" ht="20" customHeight="1">
       <x:c r="A263" s="8"/>
@@ -5882,11 +6436,13 @@
       <x:c r="L263" s="9"/>
       <x:c r="M263" s="9"/>
       <x:c r="N263" s="9"/>
-      <x:c r="O263" s="8"/>
-      <x:c r="P263" s="8"/>
+      <x:c r="O263" s="9"/>
+      <x:c r="P263" s="9"/>
       <x:c r="Q263" s="8"/>
       <x:c r="R263" s="8"/>
       <x:c r="S263" s="8"/>
+      <x:c r="T263" s="8"/>
+      <x:c r="U263" s="8"/>
     </x:row>
     <x:row r="264" ht="20" customHeight="1">
       <x:c r="A264" s="8"/>
@@ -5903,11 +6459,13 @@
       <x:c r="L264" s="9"/>
       <x:c r="M264" s="9"/>
       <x:c r="N264" s="9"/>
-      <x:c r="O264" s="8"/>
-      <x:c r="P264" s="8"/>
+      <x:c r="O264" s="9"/>
+      <x:c r="P264" s="9"/>
       <x:c r="Q264" s="8"/>
       <x:c r="R264" s="8"/>
       <x:c r="S264" s="8"/>
+      <x:c r="T264" s="8"/>
+      <x:c r="U264" s="8"/>
     </x:row>
     <x:row r="265" ht="20" customHeight="1">
       <x:c r="A265" s="8"/>
@@ -5924,11 +6482,13 @@
       <x:c r="L265" s="9"/>
       <x:c r="M265" s="9"/>
       <x:c r="N265" s="9"/>
-      <x:c r="O265" s="8"/>
-      <x:c r="P265" s="8"/>
+      <x:c r="O265" s="9"/>
+      <x:c r="P265" s="9"/>
       <x:c r="Q265" s="8"/>
       <x:c r="R265" s="8"/>
       <x:c r="S265" s="8"/>
+      <x:c r="T265" s="8"/>
+      <x:c r="U265" s="8"/>
     </x:row>
     <x:row r="266" ht="20" customHeight="1">
       <x:c r="A266" s="8"/>
@@ -5945,11 +6505,13 @@
       <x:c r="L266" s="9"/>
       <x:c r="M266" s="9"/>
       <x:c r="N266" s="9"/>
-      <x:c r="O266" s="8"/>
-      <x:c r="P266" s="8"/>
+      <x:c r="O266" s="9"/>
+      <x:c r="P266" s="9"/>
       <x:c r="Q266" s="8"/>
       <x:c r="R266" s="8"/>
       <x:c r="S266" s="8"/>
+      <x:c r="T266" s="8"/>
+      <x:c r="U266" s="8"/>
     </x:row>
     <x:row r="267" ht="20" customHeight="1">
       <x:c r="A267" s="8"/>
@@ -5966,11 +6528,13 @@
       <x:c r="L267" s="9"/>
       <x:c r="M267" s="9"/>
       <x:c r="N267" s="9"/>
-      <x:c r="O267" s="8"/>
-      <x:c r="P267" s="8"/>
+      <x:c r="O267" s="9"/>
+      <x:c r="P267" s="9"/>
       <x:c r="Q267" s="8"/>
       <x:c r="R267" s="8"/>
       <x:c r="S267" s="8"/>
+      <x:c r="T267" s="8"/>
+      <x:c r="U267" s="8"/>
     </x:row>
     <x:row r="268" ht="20" customHeight="1">
       <x:c r="A268" s="8"/>
@@ -5987,11 +6551,13 @@
       <x:c r="L268" s="9"/>
       <x:c r="M268" s="9"/>
       <x:c r="N268" s="9"/>
-      <x:c r="O268" s="8"/>
-      <x:c r="P268" s="8"/>
+      <x:c r="O268" s="9"/>
+      <x:c r="P268" s="9"/>
       <x:c r="Q268" s="8"/>
       <x:c r="R268" s="8"/>
       <x:c r="S268" s="8"/>
+      <x:c r="T268" s="8"/>
+      <x:c r="U268" s="8"/>
     </x:row>
     <x:row r="269" ht="20" customHeight="1">
       <x:c r="A269" s="8"/>
@@ -6008,11 +6574,13 @@
       <x:c r="L269" s="9"/>
       <x:c r="M269" s="9"/>
       <x:c r="N269" s="9"/>
-      <x:c r="O269" s="8"/>
-      <x:c r="P269" s="8"/>
+      <x:c r="O269" s="9"/>
+      <x:c r="P269" s="9"/>
       <x:c r="Q269" s="8"/>
       <x:c r="R269" s="8"/>
       <x:c r="S269" s="8"/>
+      <x:c r="T269" s="8"/>
+      <x:c r="U269" s="8"/>
     </x:row>
     <x:row r="270" ht="20" customHeight="1">
       <x:c r="A270" s="8"/>
@@ -6029,11 +6597,13 @@
       <x:c r="L270" s="9"/>
       <x:c r="M270" s="9"/>
       <x:c r="N270" s="9"/>
-      <x:c r="O270" s="8"/>
-      <x:c r="P270" s="8"/>
+      <x:c r="O270" s="9"/>
+      <x:c r="P270" s="9"/>
       <x:c r="Q270" s="8"/>
       <x:c r="R270" s="8"/>
       <x:c r="S270" s="8"/>
+      <x:c r="T270" s="8"/>
+      <x:c r="U270" s="8"/>
     </x:row>
     <x:row r="271" ht="20" customHeight="1">
       <x:c r="A271" s="8"/>
@@ -6050,11 +6620,13 @@
       <x:c r="L271" s="9"/>
       <x:c r="M271" s="9"/>
       <x:c r="N271" s="9"/>
-      <x:c r="O271" s="8"/>
-      <x:c r="P271" s="8"/>
+      <x:c r="O271" s="9"/>
+      <x:c r="P271" s="9"/>
       <x:c r="Q271" s="8"/>
       <x:c r="R271" s="8"/>
       <x:c r="S271" s="8"/>
+      <x:c r="T271" s="8"/>
+      <x:c r="U271" s="8"/>
     </x:row>
     <x:row r="272" ht="20" customHeight="1">
       <x:c r="A272" s="8"/>
@@ -6071,11 +6643,13 @@
       <x:c r="L272" s="9"/>
       <x:c r="M272" s="9"/>
       <x:c r="N272" s="9"/>
-      <x:c r="O272" s="8"/>
-      <x:c r="P272" s="8"/>
+      <x:c r="O272" s="9"/>
+      <x:c r="P272" s="9"/>
       <x:c r="Q272" s="8"/>
       <x:c r="R272" s="8"/>
       <x:c r="S272" s="8"/>
+      <x:c r="T272" s="8"/>
+      <x:c r="U272" s="8"/>
     </x:row>
     <x:row r="273" ht="20" customHeight="1">
       <x:c r="A273" s="8"/>
@@ -6092,11 +6666,13 @@
       <x:c r="L273" s="9"/>
       <x:c r="M273" s="9"/>
       <x:c r="N273" s="9"/>
-      <x:c r="O273" s="8"/>
-      <x:c r="P273" s="8"/>
+      <x:c r="O273" s="9"/>
+      <x:c r="P273" s="9"/>
       <x:c r="Q273" s="8"/>
       <x:c r="R273" s="8"/>
       <x:c r="S273" s="8"/>
+      <x:c r="T273" s="8"/>
+      <x:c r="U273" s="8"/>
     </x:row>
     <x:row r="274" ht="20" customHeight="1">
       <x:c r="A274" s="8"/>
@@ -6113,11 +6689,13 @@
       <x:c r="L274" s="9"/>
       <x:c r="M274" s="9"/>
       <x:c r="N274" s="9"/>
-      <x:c r="O274" s="8"/>
-      <x:c r="P274" s="8"/>
+      <x:c r="O274" s="9"/>
+      <x:c r="P274" s="9"/>
       <x:c r="Q274" s="8"/>
       <x:c r="R274" s="8"/>
       <x:c r="S274" s="8"/>
+      <x:c r="T274" s="8"/>
+      <x:c r="U274" s="8"/>
     </x:row>
     <x:row r="275" ht="20" customHeight="1">
       <x:c r="A275" s="8"/>
@@ -6134,11 +6712,13 @@
       <x:c r="L275" s="9"/>
       <x:c r="M275" s="9"/>
       <x:c r="N275" s="9"/>
-      <x:c r="O275" s="8"/>
-      <x:c r="P275" s="8"/>
+      <x:c r="O275" s="9"/>
+      <x:c r="P275" s="9"/>
       <x:c r="Q275" s="8"/>
       <x:c r="R275" s="8"/>
       <x:c r="S275" s="8"/>
+      <x:c r="T275" s="8"/>
+      <x:c r="U275" s="8"/>
     </x:row>
     <x:row r="276" ht="20" customHeight="1">
       <x:c r="A276" s="8"/>
@@ -6155,11 +6735,13 @@
       <x:c r="L276" s="9"/>
       <x:c r="M276" s="9"/>
       <x:c r="N276" s="9"/>
-      <x:c r="O276" s="8"/>
-      <x:c r="P276" s="8"/>
+      <x:c r="O276" s="9"/>
+      <x:c r="P276" s="9"/>
       <x:c r="Q276" s="8"/>
       <x:c r="R276" s="8"/>
       <x:c r="S276" s="8"/>
+      <x:c r="T276" s="8"/>
+      <x:c r="U276" s="8"/>
     </x:row>
     <x:row r="277" ht="20" customHeight="1">
       <x:c r="A277" s="8"/>
@@ -6176,11 +6758,13 @@
       <x:c r="L277" s="9"/>
       <x:c r="M277" s="9"/>
       <x:c r="N277" s="9"/>
-      <x:c r="O277" s="8"/>
-      <x:c r="P277" s="8"/>
+      <x:c r="O277" s="9"/>
+      <x:c r="P277" s="9"/>
       <x:c r="Q277" s="8"/>
       <x:c r="R277" s="8"/>
       <x:c r="S277" s="8"/>
+      <x:c r="T277" s="8"/>
+      <x:c r="U277" s="8"/>
     </x:row>
     <x:row r="278" ht="20" customHeight="1">
       <x:c r="A278" s="8"/>
@@ -6197,11 +6781,13 @@
       <x:c r="L278" s="9"/>
       <x:c r="M278" s="9"/>
       <x:c r="N278" s="9"/>
-      <x:c r="O278" s="8"/>
-      <x:c r="P278" s="8"/>
+      <x:c r="O278" s="9"/>
+      <x:c r="P278" s="9"/>
       <x:c r="Q278" s="8"/>
       <x:c r="R278" s="8"/>
       <x:c r="S278" s="8"/>
+      <x:c r="T278" s="8"/>
+      <x:c r="U278" s="8"/>
     </x:row>
     <x:row r="279" ht="20" customHeight="1">
       <x:c r="A279" s="8"/>
@@ -6218,11 +6804,13 @@
       <x:c r="L279" s="9"/>
       <x:c r="M279" s="9"/>
       <x:c r="N279" s="9"/>
-      <x:c r="O279" s="8"/>
-      <x:c r="P279" s="8"/>
+      <x:c r="O279" s="9"/>
+      <x:c r="P279" s="9"/>
       <x:c r="Q279" s="8"/>
       <x:c r="R279" s="8"/>
       <x:c r="S279" s="8"/>
+      <x:c r="T279" s="8"/>
+      <x:c r="U279" s="8"/>
     </x:row>
     <x:row r="280" ht="20" customHeight="1">
       <x:c r="A280" s="8"/>
@@ -6239,11 +6827,13 @@
       <x:c r="L280" s="9"/>
       <x:c r="M280" s="9"/>
       <x:c r="N280" s="9"/>
-      <x:c r="O280" s="8"/>
-      <x:c r="P280" s="8"/>
+      <x:c r="O280" s="9"/>
+      <x:c r="P280" s="9"/>
       <x:c r="Q280" s="8"/>
       <x:c r="R280" s="8"/>
       <x:c r="S280" s="8"/>
+      <x:c r="T280" s="8"/>
+      <x:c r="U280" s="8"/>
     </x:row>
     <x:row r="281" ht="20" customHeight="1">
       <x:c r="A281" s="8"/>
@@ -6260,11 +6850,13 @@
       <x:c r="L281" s="9"/>
       <x:c r="M281" s="9"/>
       <x:c r="N281" s="9"/>
-      <x:c r="O281" s="8"/>
-      <x:c r="P281" s="8"/>
+      <x:c r="O281" s="9"/>
+      <x:c r="P281" s="9"/>
       <x:c r="Q281" s="8"/>
       <x:c r="R281" s="8"/>
       <x:c r="S281" s="8"/>
+      <x:c r="T281" s="8"/>
+      <x:c r="U281" s="8"/>
     </x:row>
     <x:row r="282" ht="20" customHeight="1">
       <x:c r="A282" s="8"/>
@@ -6281,11 +6873,13 @@
       <x:c r="L282" s="9"/>
       <x:c r="M282" s="9"/>
       <x:c r="N282" s="9"/>
-      <x:c r="O282" s="8"/>
-      <x:c r="P282" s="8"/>
+      <x:c r="O282" s="9"/>
+      <x:c r="P282" s="9"/>
       <x:c r="Q282" s="8"/>
       <x:c r="R282" s="8"/>
       <x:c r="S282" s="8"/>
+      <x:c r="T282" s="8"/>
+      <x:c r="U282" s="8"/>
     </x:row>
     <x:row r="283" ht="20" customHeight="1">
       <x:c r="A283" s="8"/>
@@ -6302,11 +6896,13 @@
       <x:c r="L283" s="9"/>
       <x:c r="M283" s="9"/>
       <x:c r="N283" s="9"/>
-      <x:c r="O283" s="8"/>
-      <x:c r="P283" s="8"/>
+      <x:c r="O283" s="9"/>
+      <x:c r="P283" s="9"/>
       <x:c r="Q283" s="8"/>
       <x:c r="R283" s="8"/>
       <x:c r="S283" s="8"/>
+      <x:c r="T283" s="8"/>
+      <x:c r="U283" s="8"/>
     </x:row>
     <x:row r="284" ht="20" customHeight="1">
       <x:c r="A284" s="8"/>
@@ -6323,11 +6919,13 @@
       <x:c r="L284" s="9"/>
       <x:c r="M284" s="9"/>
       <x:c r="N284" s="9"/>
-      <x:c r="O284" s="8"/>
-      <x:c r="P284" s="8"/>
+      <x:c r="O284" s="9"/>
+      <x:c r="P284" s="9"/>
       <x:c r="Q284" s="8"/>
       <x:c r="R284" s="8"/>
       <x:c r="S284" s="8"/>
+      <x:c r="T284" s="8"/>
+      <x:c r="U284" s="8"/>
     </x:row>
     <x:row r="285" ht="20" customHeight="1">
       <x:c r="A285" s="8"/>
@@ -6344,11 +6942,13 @@
       <x:c r="L285" s="9"/>
       <x:c r="M285" s="9"/>
       <x:c r="N285" s="9"/>
-      <x:c r="O285" s="8"/>
-      <x:c r="P285" s="8"/>
+      <x:c r="O285" s="9"/>
+      <x:c r="P285" s="9"/>
       <x:c r="Q285" s="8"/>
       <x:c r="R285" s="8"/>
       <x:c r="S285" s="8"/>
+      <x:c r="T285" s="8"/>
+      <x:c r="U285" s="8"/>
     </x:row>
     <x:row r="286" ht="20" customHeight="1">
       <x:c r="A286" s="8"/>
@@ -6365,11 +6965,13 @@
       <x:c r="L286" s="9"/>
       <x:c r="M286" s="9"/>
       <x:c r="N286" s="9"/>
-      <x:c r="O286" s="8"/>
-      <x:c r="P286" s="8"/>
+      <x:c r="O286" s="9"/>
+      <x:c r="P286" s="9"/>
       <x:c r="Q286" s="8"/>
       <x:c r="R286" s="8"/>
       <x:c r="S286" s="8"/>
+      <x:c r="T286" s="8"/>
+      <x:c r="U286" s="8"/>
     </x:row>
     <x:row r="287" ht="20" customHeight="1">
       <x:c r="A287" s="8"/>
@@ -6386,11 +6988,13 @@
       <x:c r="L287" s="9"/>
       <x:c r="M287" s="9"/>
       <x:c r="N287" s="9"/>
-      <x:c r="O287" s="8"/>
-      <x:c r="P287" s="8"/>
+      <x:c r="O287" s="9"/>
+      <x:c r="P287" s="9"/>
       <x:c r="Q287" s="8"/>
       <x:c r="R287" s="8"/>
       <x:c r="S287" s="8"/>
+      <x:c r="T287" s="8"/>
+      <x:c r="U287" s="8"/>
     </x:row>
     <x:row r="288" ht="20" customHeight="1">
       <x:c r="A288" s="8"/>
@@ -6407,11 +7011,13 @@
       <x:c r="L288" s="9"/>
       <x:c r="M288" s="9"/>
       <x:c r="N288" s="9"/>
-      <x:c r="O288" s="8"/>
-      <x:c r="P288" s="8"/>
+      <x:c r="O288" s="9"/>
+      <x:c r="P288" s="9"/>
       <x:c r="Q288" s="8"/>
       <x:c r="R288" s="8"/>
       <x:c r="S288" s="8"/>
+      <x:c r="T288" s="8"/>
+      <x:c r="U288" s="8"/>
     </x:row>
     <x:row r="289" ht="20" customHeight="1">
       <x:c r="A289" s="8"/>
@@ -6428,11 +7034,13 @@
       <x:c r="L289" s="9"/>
       <x:c r="M289" s="9"/>
       <x:c r="N289" s="9"/>
-      <x:c r="O289" s="8"/>
-      <x:c r="P289" s="8"/>
+      <x:c r="O289" s="9"/>
+      <x:c r="P289" s="9"/>
       <x:c r="Q289" s="8"/>
       <x:c r="R289" s="8"/>
       <x:c r="S289" s="8"/>
+      <x:c r="T289" s="8"/>
+      <x:c r="U289" s="8"/>
     </x:row>
     <x:row r="290" ht="20" customHeight="1">
       <x:c r="A290" s="8"/>
@@ -6449,11 +7057,13 @@
       <x:c r="L290" s="9"/>
       <x:c r="M290" s="9"/>
       <x:c r="N290" s="9"/>
-      <x:c r="O290" s="8"/>
-      <x:c r="P290" s="8"/>
+      <x:c r="O290" s="9"/>
+      <x:c r="P290" s="9"/>
       <x:c r="Q290" s="8"/>
       <x:c r="R290" s="8"/>
       <x:c r="S290" s="8"/>
+      <x:c r="T290" s="8"/>
+      <x:c r="U290" s="8"/>
     </x:row>
     <x:row r="291" ht="20" customHeight="1">
       <x:c r="A291" s="8"/>
@@ -6470,11 +7080,13 @@
       <x:c r="L291" s="9"/>
       <x:c r="M291" s="9"/>
       <x:c r="N291" s="9"/>
-      <x:c r="O291" s="8"/>
-      <x:c r="P291" s="8"/>
+      <x:c r="O291" s="9"/>
+      <x:c r="P291" s="9"/>
       <x:c r="Q291" s="8"/>
       <x:c r="R291" s="8"/>
       <x:c r="S291" s="8"/>
+      <x:c r="T291" s="8"/>
+      <x:c r="U291" s="8"/>
     </x:row>
     <x:row r="292" ht="20" customHeight="1">
       <x:c r="A292" s="8"/>
@@ -6491,11 +7103,13 @@
       <x:c r="L292" s="9"/>
       <x:c r="M292" s="9"/>
       <x:c r="N292" s="9"/>
-      <x:c r="O292" s="8"/>
-      <x:c r="P292" s="8"/>
+      <x:c r="O292" s="9"/>
+      <x:c r="P292" s="9"/>
       <x:c r="Q292" s="8"/>
       <x:c r="R292" s="8"/>
       <x:c r="S292" s="8"/>
+      <x:c r="T292" s="8"/>
+      <x:c r="U292" s="8"/>
     </x:row>
     <x:row r="293" ht="20" customHeight="1">
       <x:c r="A293" s="8"/>
@@ -6512,11 +7126,13 @@
       <x:c r="L293" s="9"/>
       <x:c r="M293" s="9"/>
       <x:c r="N293" s="9"/>
-      <x:c r="O293" s="8"/>
-      <x:c r="P293" s="8"/>
+      <x:c r="O293" s="9"/>
+      <x:c r="P293" s="9"/>
       <x:c r="Q293" s="8"/>
       <x:c r="R293" s="8"/>
       <x:c r="S293" s="8"/>
+      <x:c r="T293" s="8"/>
+      <x:c r="U293" s="8"/>
     </x:row>
     <x:row r="294" ht="20" customHeight="1">
       <x:c r="A294" s="8"/>
@@ -6533,11 +7149,13 @@
       <x:c r="L294" s="9"/>
       <x:c r="M294" s="9"/>
       <x:c r="N294" s="9"/>
-      <x:c r="O294" s="8"/>
-      <x:c r="P294" s="8"/>
+      <x:c r="O294" s="9"/>
+      <x:c r="P294" s="9"/>
       <x:c r="Q294" s="8"/>
       <x:c r="R294" s="8"/>
       <x:c r="S294" s="8"/>
+      <x:c r="T294" s="8"/>
+      <x:c r="U294" s="8"/>
     </x:row>
     <x:row r="295" ht="20" customHeight="1">
       <x:c r="A295" s="8"/>
@@ -6554,11 +7172,13 @@
       <x:c r="L295" s="9"/>
       <x:c r="M295" s="9"/>
       <x:c r="N295" s="9"/>
-      <x:c r="O295" s="8"/>
-      <x:c r="P295" s="8"/>
+      <x:c r="O295" s="9"/>
+      <x:c r="P295" s="9"/>
       <x:c r="Q295" s="8"/>
       <x:c r="R295" s="8"/>
       <x:c r="S295" s="8"/>
+      <x:c r="T295" s="8"/>
+      <x:c r="U295" s="8"/>
     </x:row>
     <x:row r="296" ht="20" customHeight="1">
       <x:c r="A296" s="8"/>
@@ -6575,11 +7195,13 @@
       <x:c r="L296" s="9"/>
       <x:c r="M296" s="9"/>
       <x:c r="N296" s="9"/>
-      <x:c r="O296" s="8"/>
-      <x:c r="P296" s="8"/>
+      <x:c r="O296" s="9"/>
+      <x:c r="P296" s="9"/>
       <x:c r="Q296" s="8"/>
       <x:c r="R296" s="8"/>
       <x:c r="S296" s="8"/>
+      <x:c r="T296" s="8"/>
+      <x:c r="U296" s="8"/>
     </x:row>
     <x:row r="297" ht="20" customHeight="1">
       <x:c r="A297" s="8"/>
@@ -6596,11 +7218,13 @@
       <x:c r="L297" s="9"/>
       <x:c r="M297" s="9"/>
       <x:c r="N297" s="9"/>
-      <x:c r="O297" s="8"/>
-      <x:c r="P297" s="8"/>
+      <x:c r="O297" s="9"/>
+      <x:c r="P297" s="9"/>
       <x:c r="Q297" s="8"/>
       <x:c r="R297" s="8"/>
       <x:c r="S297" s="8"/>
+      <x:c r="T297" s="8"/>
+      <x:c r="U297" s="8"/>
     </x:row>
     <x:row r="298" ht="20" customHeight="1">
       <x:c r="A298" s="8"/>
@@ -6617,11 +7241,13 @@
       <x:c r="L298" s="9"/>
       <x:c r="M298" s="9"/>
       <x:c r="N298" s="9"/>
-      <x:c r="O298" s="8"/>
-      <x:c r="P298" s="8"/>
+      <x:c r="O298" s="9"/>
+      <x:c r="P298" s="9"/>
       <x:c r="Q298" s="8"/>
       <x:c r="R298" s="8"/>
       <x:c r="S298" s="8"/>
+      <x:c r="T298" s="8"/>
+      <x:c r="U298" s="8"/>
     </x:row>
     <x:row r="299" ht="20" customHeight="1">
       <x:c r="A299" s="8"/>
@@ -6638,11 +7264,13 @@
       <x:c r="L299" s="9"/>
       <x:c r="M299" s="9"/>
       <x:c r="N299" s="9"/>
-      <x:c r="O299" s="8"/>
-      <x:c r="P299" s="8"/>
+      <x:c r="O299" s="9"/>
+      <x:c r="P299" s="9"/>
       <x:c r="Q299" s="8"/>
       <x:c r="R299" s="8"/>
       <x:c r="S299" s="8"/>
+      <x:c r="T299" s="8"/>
+      <x:c r="U299" s="8"/>
     </x:row>
     <x:row r="300" ht="20" customHeight="1">
       <x:c r="A300" s="8"/>
@@ -6659,11 +7287,13 @@
       <x:c r="L300" s="9"/>
       <x:c r="M300" s="9"/>
       <x:c r="N300" s="9"/>
-      <x:c r="O300" s="8"/>
-      <x:c r="P300" s="8"/>
+      <x:c r="O300" s="9"/>
+      <x:c r="P300" s="9"/>
       <x:c r="Q300" s="8"/>
       <x:c r="R300" s="8"/>
       <x:c r="S300" s="8"/>
+      <x:c r="T300" s="8"/>
+      <x:c r="U300" s="8"/>
     </x:row>
     <x:row r="301" ht="20" customHeight="1">
       <x:c r="A301" s="8"/>
@@ -6680,11 +7310,13 @@
       <x:c r="L301" s="9"/>
       <x:c r="M301" s="9"/>
       <x:c r="N301" s="9"/>
-      <x:c r="O301" s="8"/>
-      <x:c r="P301" s="8"/>
+      <x:c r="O301" s="9"/>
+      <x:c r="P301" s="9"/>
       <x:c r="Q301" s="8"/>
       <x:c r="R301" s="8"/>
       <x:c r="S301" s="8"/>
+      <x:c r="T301" s="8"/>
+      <x:c r="U301" s="8"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6714,7 +7346,7 @@
         <x:v>Wymagane pola</x:v>
       </x:c>
       <x:c r="B3" s="13" t="str">
-        <x:v>Nazwa urządzenia, znak wytwórczy i numer fabryczny.</x:v>
+        <x:v>Nazwa urządzenia, nazwa lub znak wytwórcy i numer fabryczny.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">

</xml_diff>